<commit_message>
predm parse criterion, pp out of preds/a
</commit_message>
<xml_diff>
--- a/src/sastadev/data/methods/TARSP_Index_Current.xlsx
+++ b/src/sastadev/data/methods/TARSP_Index_Current.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\jodijk\myprograms\python\sastacode\mysastadev\src\sastadev\data\methods\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAE459F3-262A-4509-8E0D-21BCCE176804}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55B4D02E-2B97-40AA-AFB4-0343EF2A321C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1865,9 +1865,6 @@
     <t>//node[ @lemma="niets" or @lemma="niks" or @lemma="zelf"]</t>
   </si>
   <si>
-    <t>tarsp2017,auris</t>
-  </si>
-  <si>
     <t>taalmaat is veranderd in 2017; vgl T085</t>
   </si>
   <si>
@@ -1893,9 +1890,6 @@
   </si>
   <si>
     <t>//node[%BezZn%]</t>
-  </si>
-  <si>
-    <t>//node[@pt="n" and %realwordnode% and @lemma!="kijk" and %thisistheonlyrealword%]</t>
   </si>
   <si>
     <t>// node[@rel="mod" and @cat="pp" and parent::node[@cat="np" and node[@rel="hd" and @pt!="ww"]] and @begin &gt;= ../node[@rel="hd"]/@end]</t>
@@ -1922,6 +1916,12 @@
   </si>
   <si>
     <t>//node[@lemma="alles"  or @lemma="niets" or @lemma="niks" or %zelfst_wat% or (@lemma="u" and not(../node[%dankje_VU%])) or @lemma="ons"  or @lemma="zelf"]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dir </t>
+  </si>
+  <si>
+    <t>//node[(@pt="n" or @pt="tw") and %realwordnode% and @lemma!="kijk" and %thisistheonlyrealword%]</t>
   </si>
 </sst>
 </file>
@@ -2730,7 +2730,7 @@
         <v>6</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="L9" s="2" t="s">
         <v>353</v>
@@ -2844,7 +2844,7 @@
         <v>3</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="L12" s="2" t="s">
         <v>353</v>
@@ -2879,7 +2879,7 @@
         <v>5</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="L13" s="3" t="s">
         <v>353</v>
@@ -2952,7 +2952,7 @@
         <v>4</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="L15" s="2" t="s">
         <v>353</v>
@@ -3092,7 +3092,7 @@
         <v>1</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="L19" s="2" t="s">
         <v>353</v>
@@ -3159,7 +3159,7 @@
         <v>4</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="L21" s="2" t="s">
         <v>353</v>
@@ -3457,7 +3457,7 @@
         <v>2</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="L29" s="2" t="s">
         <v>353</v>
@@ -4036,7 +4036,7 @@
         <v>3</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="L44" s="2" t="s">
         <v>353</v>
@@ -4360,7 +4360,7 @@
         <v>6</v>
       </c>
       <c r="K53" s="2" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="L53" s="2" t="s">
         <v>353</v>
@@ -5387,7 +5387,7 @@
         <v>6</v>
       </c>
       <c r="K79" s="2" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="L79" s="2" t="s">
         <v>353</v>
@@ -5463,7 +5463,7 @@
         <v>4</v>
       </c>
       <c r="K81" s="3" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="L81" s="3" t="s">
         <v>353</v>
@@ -6526,7 +6526,7 @@
         <v>7</v>
       </c>
       <c r="K110" s="9" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="L110" s="10" t="s">
         <v>353</v>
@@ -6708,7 +6708,7 @@
         <v>1</v>
       </c>
       <c r="K115" s="3" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="L115" s="3" t="s">
         <v>353</v>
@@ -7626,7 +7626,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="140" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A140" s="2" t="s">
         <v>350</v>
       </c>
@@ -7652,7 +7652,7 @@
         <v>1</v>
       </c>
       <c r="K140" s="3" t="s">
-        <v>604</v>
+        <v>610</v>
       </c>
       <c r="L140" s="2" t="s">
         <v>353</v>
@@ -7929,7 +7929,7 @@
         <v>411</v>
       </c>
       <c r="K148" s="2" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="L148" s="2" t="s">
         <v>353</v>
@@ -8197,10 +8197,10 @@
         <v>441</v>
       </c>
       <c r="R156" s="2" t="s">
+        <v>609</v>
+      </c>
+      <c r="U156" s="2" t="s">
         <v>594</v>
-      </c>
-      <c r="U156" s="2" t="s">
-        <v>595</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ga imperative anv vcw updates
</commit_message>
<xml_diff>
--- a/src/sastadev/data/methods/TARSP_Index_Current.xlsx
+++ b/src/sastadev/data/methods/TARSP_Index_Current.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\jodijk\myprograms\python\sastacode\mysastadev\src\sastadev\data\methods\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55B4D02E-2B97-40AA-AFB4-0343EF2A321C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C77A5523-285A-4E3C-B89C-7BE63E2857F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1159,12 +1159,6 @@
     <t>PV-loos</t>
   </si>
   <si>
-    <t>//node[@cat="np" and node[@pt="n" and @rel="hd"] and node[@pt="vnw" and @vwtype="aanw" and @rel="det" and (@lemma="die" or @lemma="deze")] and count(node)=2]</t>
-  </si>
-  <si>
-    <t>//node[@cat="np" and node[@pt="n" and @rel="hd"] and node[@pt="vnw" and @vwtype="aanw" and @rel="det" and (@lemma="dit" or @lemma="dat")] and count(node)=2]</t>
-  </si>
-  <si>
     <t>removed @pt=vwn because that only occurs as 'ene' or in een en ander.</t>
   </si>
   <si>
@@ -1875,9 +1869,6 @@
   </si>
   <si>
     <t xml:space="preserve">//node[%bvb% ] </t>
-  </si>
-  <si>
-    <t>//node[@rel="mod"and @cat="cp" and not(%Tarsp_ofmod%) and  node[@rel="body" and node[@pt="ww" and @pvagr and @rel="hd"]]]</t>
   </si>
   <si>
     <t>//node[%BepBvZn%]</t>
@@ -1922,6 +1913,16 @@
   </si>
   <si>
     <t>//node[(@pt="n" or @pt="tw") and %realwordnode% and @lemma!="kijk" and %thisistheonlyrealword%]</t>
+  </si>
+  <si>
+    <t>//node[(@rel="mod" or @rel="dp")  and @cat="cp" and not(%Tarsp_ofmod%) and  not(%Tarsp_datmod%) and node[@rel="body" and node[@pt="ww" and @pvagr and @rel="hd"]]]</t>
+  </si>
+  <si>
+    <t>//node[@cat="np" and node[(@pt="n" or %substantivised_nphead%)  and @rel="hd"] and node[@pt="vnw" and @vwtype="aanw" and @rel="det" and (@lemma="dit" or @lemma="dat")] and count(node)=2]</t>
+  </si>
+  <si>
+    <t>//node[@cat="np" and node[(@pt="n" or %substantivised_nphead%) and @rel="hd"] and node[@pt="vnw" and @vwtype="aanw" and @rel="det" and (@lemma="die" or @lemma="deze")] and 
+count(node)=2]</t>
   </si>
 </sst>
 </file>
@@ -2393,31 +2394,31 @@
         <v>157</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="P1" s="1" t="s">
+        <v>545</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>546</v>
+      </c>
+      <c r="R1" s="1" t="s">
         <v>547</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>548</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>549</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>550</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>551</v>
       </c>
       <c r="U1" s="1" t="s">
         <v>158</v>
@@ -2437,13 +2438,13 @@
         <v>193</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>70</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>353</v>
@@ -2455,7 +2456,7 @@
         <v>3</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>353</v>
@@ -2464,10 +2465,10 @@
         <v>354</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.3">
@@ -2496,7 +2497,7 @@
         <v>6</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="L3" s="2" t="s">
         <v>353</v>
@@ -2505,10 +2506,10 @@
         <v>353</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U3" s="2" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.3">
@@ -2525,7 +2526,7 @@
         <v>193</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>63</v>
@@ -2546,10 +2547,10 @@
         <v>354</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="R4" s="2" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.3">
@@ -2584,7 +2585,7 @@
         <v>354</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U5" s="2" t="s">
         <v>185</v>
@@ -2613,7 +2614,7 @@
         <v>1</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>353</v>
@@ -2622,13 +2623,13 @@
         <v>354</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U6" s="2" t="s">
         <v>359</v>
       </c>
       <c r="V6" s="2" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="7" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
@@ -2642,7 +2643,7 @@
         <v>193</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>353</v>
@@ -2654,7 +2655,7 @@
         <v>1</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="L7" s="2" t="s">
         <v>354</v>
@@ -2663,7 +2664,7 @@
         <v>354</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="8" spans="1:22" ht="115.2" hidden="1" x14ac:dyDescent="0.3">
@@ -2692,7 +2693,7 @@
         <v>4</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="L8" s="3" t="s">
         <v>354</v>
@@ -2701,7 +2702,7 @@
         <v>354</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.3">
@@ -2730,7 +2731,7 @@
         <v>6</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>598</v>
+        <v>608</v>
       </c>
       <c r="L9" s="2" t="s">
         <v>353</v>
@@ -2739,10 +2740,10 @@
         <v>353</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U9" s="2" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
     <row r="10" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
@@ -2768,7 +2769,7 @@
         <v>4</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="L10" s="3" t="s">
         <v>353</v>
@@ -2777,7 +2778,7 @@
         <v>354</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="11" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
@@ -2812,7 +2813,7 @@
         <v>354</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.3">
@@ -2832,7 +2833,7 @@
         <v>38</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>353</v>
@@ -2844,7 +2845,7 @@
         <v>3</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="L12" s="2" t="s">
         <v>353</v>
@@ -2853,7 +2854,7 @@
         <v>354</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.3">
@@ -2879,7 +2880,7 @@
         <v>5</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
       <c r="L13" s="3" t="s">
         <v>353</v>
@@ -2888,7 +2889,7 @@
         <v>354</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
@@ -2917,7 +2918,7 @@
         <v>4</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="L14" s="2" t="s">
         <v>354</v>
@@ -2926,7 +2927,7 @@
         <v>354</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="15" spans="1:22" x14ac:dyDescent="0.3">
@@ -2952,7 +2953,7 @@
         <v>4</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="L15" s="2" t="s">
         <v>353</v>
@@ -2961,7 +2962,7 @@
         <v>354</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
@@ -2981,7 +2982,7 @@
         <v>353</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="L16" s="2" t="s">
         <v>354</v>
@@ -2990,7 +2991,7 @@
         <v>354</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="17" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
@@ -3022,7 +3023,7 @@
         <v>353</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.3">
@@ -3039,10 +3040,10 @@
         <v>193</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="H18" s="2" t="s">
         <v>353</v>
@@ -3060,10 +3061,10 @@
         <v>354</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="P18" s="2" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.3">
@@ -3077,10 +3078,10 @@
         <v>193</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>353</v>
@@ -3092,7 +3093,7 @@
         <v>1</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="L19" s="2" t="s">
         <v>353</v>
@@ -3101,7 +3102,7 @@
         <v>353</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.3">
@@ -3133,7 +3134,7 @@
         <v>354</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.3">
@@ -3159,7 +3160,7 @@
         <v>4</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="L21" s="2" t="s">
         <v>353</v>
@@ -3168,7 +3169,7 @@
         <v>354</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.3">
@@ -3194,7 +3195,7 @@
         <v>3</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="L22" s="2" t="s">
         <v>353</v>
@@ -3203,7 +3204,7 @@
         <v>354</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.3">
@@ -3223,7 +3224,7 @@
         <v>47</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="H23" s="2" t="s">
         <v>353</v>
@@ -3235,7 +3236,7 @@
         <v>5</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="L23" s="2" t="s">
         <v>353</v>
@@ -3244,7 +3245,7 @@
         <v>354</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="24" spans="1:21" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -3261,13 +3262,13 @@
         <v>193</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>26</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="H24" s="2" t="s">
         <v>353</v>
@@ -3279,7 +3280,7 @@
         <v>2</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="L24" s="2" t="s">
         <v>353</v>
@@ -3288,10 +3289,10 @@
         <v>354</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U24" s="3" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
     </row>
     <row r="25" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
@@ -3323,7 +3324,7 @@
         <v>354</v>
       </c>
       <c r="N25" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="26" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
@@ -3349,7 +3350,7 @@
         <v>4</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="L26" s="3" t="s">
         <v>353</v>
@@ -3358,13 +3359,13 @@
         <v>354</v>
       </c>
       <c r="N26" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U26" s="2" t="s">
-        <v>475</v>
-      </c>
-    </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.3">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="27" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>238</v>
       </c>
@@ -3386,8 +3387,8 @@
       <c r="J27" s="2">
         <v>4</v>
       </c>
-      <c r="K27" s="2" t="s">
-        <v>369</v>
+      <c r="K27" s="3" t="s">
+        <v>610</v>
       </c>
       <c r="L27" s="2" t="s">
         <v>353</v>
@@ -3396,7 +3397,7 @@
         <v>354</v>
       </c>
       <c r="N27" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.3">
@@ -3422,7 +3423,7 @@
         <v>5</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>370</v>
+        <v>609</v>
       </c>
       <c r="L28" s="2" t="s">
         <v>353</v>
@@ -3431,7 +3432,7 @@
         <v>353</v>
       </c>
       <c r="N28" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.3">
@@ -3457,7 +3458,7 @@
         <v>2</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="L29" s="2" t="s">
         <v>353</v>
@@ -3466,10 +3467,10 @@
         <v>354</v>
       </c>
       <c r="N29" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U29" s="2" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.3">
@@ -3495,7 +3496,7 @@
         <v>3</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="L30" s="2" t="s">
         <v>353</v>
@@ -3504,7 +3505,7 @@
         <v>353</v>
       </c>
       <c r="N30" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U30" s="2" t="s">
         <v>185</v>
@@ -3542,10 +3543,10 @@
         <v>354</v>
       </c>
       <c r="N31" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="R31" s="2" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
     </row>
     <row r="32" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
@@ -3583,7 +3584,7 @@
         <v>354</v>
       </c>
       <c r="N32" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.3">
@@ -3615,7 +3616,7 @@
         <v>3</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="L33" s="2" t="s">
         <v>353</v>
@@ -3624,10 +3625,10 @@
         <v>354</v>
       </c>
       <c r="N33" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="R33" s="2" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.3">
@@ -3653,7 +3654,7 @@
         <v>6</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="L34" s="2" t="s">
         <v>353</v>
@@ -3662,7 +3663,7 @@
         <v>354</v>
       </c>
       <c r="N34" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.3">
@@ -3697,7 +3698,7 @@
         <v>353</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="36" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
@@ -3732,7 +3733,7 @@
         <v>353</v>
       </c>
       <c r="N36" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.3">
@@ -3758,7 +3759,7 @@
         <v>3</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="L37" s="2" t="s">
         <v>353</v>
@@ -3767,7 +3768,7 @@
         <v>354</v>
       </c>
       <c r="N37" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.3">
@@ -3787,7 +3788,7 @@
         <v>209</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="H38" s="2" t="s">
         <v>353</v>
@@ -3799,7 +3800,7 @@
         <v>363</v>
       </c>
       <c r="K38" s="3" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="L38" s="3" t="s">
         <v>353</v>
@@ -3808,7 +3809,7 @@
         <v>354</v>
       </c>
       <c r="N38" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.3">
@@ -3828,7 +3829,7 @@
         <v>210</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="H39" s="2" t="s">
         <v>353</v>
@@ -3840,7 +3841,7 @@
         <v>4</v>
       </c>
       <c r="K39" s="3" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="L39" s="3" t="s">
         <v>353</v>
@@ -3849,7 +3850,7 @@
         <v>354</v>
       </c>
       <c r="N39" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.3">
@@ -3866,7 +3867,7 @@
         <v>145</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="H40" s="2" t="s">
         <v>353</v>
@@ -3878,7 +3879,7 @@
         <v>3</v>
       </c>
       <c r="K40" s="3" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="L40" s="3" t="s">
         <v>353</v>
@@ -3887,10 +3888,10 @@
         <v>353</v>
       </c>
       <c r="N40" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U40" s="2" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.3">
@@ -3925,7 +3926,7 @@
         <v>353</v>
       </c>
       <c r="N41" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.3">
@@ -3945,7 +3946,7 @@
         <v>67</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="H42" s="2" t="s">
         <v>353</v>
@@ -3963,7 +3964,7 @@
         <v>354</v>
       </c>
       <c r="N42" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U42" s="2" t="s">
         <v>161</v>
@@ -3983,10 +3984,10 @@
         <v>193</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="H43" s="2" t="s">
         <v>353</v>
@@ -3998,7 +3999,7 @@
         <v>3</v>
       </c>
       <c r="K43" s="3" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="L43" s="2" t="s">
         <v>353</v>
@@ -4007,7 +4008,7 @@
         <v>354</v>
       </c>
       <c r="N43" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U43" s="2" t="s">
         <v>358</v>
@@ -4036,7 +4037,7 @@
         <v>3</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>607</v>
+        <v>604</v>
       </c>
       <c r="L44" s="2" t="s">
         <v>353</v>
@@ -4045,7 +4046,7 @@
         <v>354</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="45" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
@@ -4071,7 +4072,7 @@
         <v>6</v>
       </c>
       <c r="K45" s="3" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="L45" s="2" t="s">
         <v>353</v>
@@ -4080,7 +4081,7 @@
         <v>354</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.3">
@@ -4103,7 +4104,7 @@
         <v>202</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="H46" s="2" t="s">
         <v>353</v>
@@ -4115,7 +4116,7 @@
         <v>2</v>
       </c>
       <c r="K46" s="2" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="L46" s="2" t="s">
         <v>353</v>
@@ -4124,7 +4125,7 @@
         <v>354</v>
       </c>
       <c r="N46" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="47" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
@@ -4150,7 +4151,7 @@
         <v>6</v>
       </c>
       <c r="K47" s="3" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="L47" s="2" t="s">
         <v>353</v>
@@ -4159,7 +4160,7 @@
         <v>354</v>
       </c>
       <c r="N47" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U47" s="2" t="s">
         <v>185</v>
@@ -4179,7 +4180,7 @@
         <v>354</v>
       </c>
       <c r="K48" s="3" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="L48" s="3" t="s">
         <v>354</v>
@@ -4188,7 +4189,7 @@
         <v>354</v>
       </c>
       <c r="N48" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U48" s="6" t="s">
         <v>180</v>
@@ -4226,7 +4227,7 @@
         <v>354</v>
       </c>
       <c r="N49" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="50" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
@@ -4252,7 +4253,7 @@
         <v>5</v>
       </c>
       <c r="K50" s="3" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="L50" s="2" t="s">
         <v>353</v>
@@ -4261,7 +4262,7 @@
         <v>354</v>
       </c>
       <c r="N50" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.3">
@@ -4287,7 +4288,7 @@
         <v>4</v>
       </c>
       <c r="K51" s="2" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="L51" s="2" t="s">
         <v>353</v>
@@ -4296,7 +4297,7 @@
         <v>354</v>
       </c>
       <c r="N51" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.3">
@@ -4325,7 +4326,7 @@
         <v>2</v>
       </c>
       <c r="K52" s="2" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="L52" s="2" t="s">
         <v>353</v>
@@ -4334,7 +4335,7 @@
         <v>354</v>
       </c>
       <c r="N52" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.3">
@@ -4360,7 +4361,7 @@
         <v>6</v>
       </c>
       <c r="K53" s="2" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="L53" s="2" t="s">
         <v>353</v>
@@ -4369,7 +4370,7 @@
         <v>354</v>
       </c>
       <c r="N53" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.3">
@@ -4398,7 +4399,7 @@
         <v>6</v>
       </c>
       <c r="K54" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="L54" s="2" t="s">
         <v>353</v>
@@ -4407,7 +4408,7 @@
         <v>354</v>
       </c>
       <c r="N54" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="55" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
@@ -4442,7 +4443,7 @@
         <v>353</v>
       </c>
       <c r="N55" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.3">
@@ -4474,10 +4475,10 @@
         <v>354</v>
       </c>
       <c r="N56" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="R56" s="2" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
     </row>
     <row r="57" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
@@ -4503,7 +4504,7 @@
         <v>1</v>
       </c>
       <c r="K57" s="3" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="L57" s="2" t="s">
         <v>354</v>
@@ -4512,7 +4513,7 @@
         <v>354</v>
       </c>
       <c r="N57" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.3">
@@ -4532,7 +4533,7 @@
         <v>21</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="H58" s="2" t="s">
         <v>353</v>
@@ -4544,7 +4545,7 @@
         <v>2</v>
       </c>
       <c r="K58" s="2" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="L58" s="2" t="s">
         <v>353</v>
@@ -4553,7 +4554,7 @@
         <v>353</v>
       </c>
       <c r="N58" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.3">
@@ -4573,7 +4574,7 @@
         <v>39</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="H59" s="2" t="s">
         <v>353</v>
@@ -4585,7 +4586,7 @@
         <v>3</v>
       </c>
       <c r="K59" s="2" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="L59" s="2" t="s">
         <v>353</v>
@@ -4594,7 +4595,7 @@
         <v>354</v>
       </c>
       <c r="N59" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.3">
@@ -4611,7 +4612,7 @@
         <v>193</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="F60" s="2" t="s">
         <v>65</v>
@@ -4632,10 +4633,10 @@
         <v>354</v>
       </c>
       <c r="N60" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="R60" s="2" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
     </row>
     <row r="61" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
@@ -4670,10 +4671,10 @@
         <v>354</v>
       </c>
       <c r="N61" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U61" s="2" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
     </row>
     <row r="62" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
@@ -4708,10 +4709,10 @@
         <v>354</v>
       </c>
       <c r="N62" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U62" s="2" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="63" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
@@ -4746,10 +4747,10 @@
         <v>354</v>
       </c>
       <c r="N63" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U63" s="2" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
     </row>
     <row r="64" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
@@ -4775,7 +4776,7 @@
         <v>4</v>
       </c>
       <c r="K64" s="2" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="L64" s="2" t="s">
         <v>354</v>
@@ -4784,7 +4785,7 @@
         <v>353</v>
       </c>
       <c r="N64" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.3">
@@ -4816,7 +4817,7 @@
         <v>2</v>
       </c>
       <c r="K65" s="2" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="L65" s="2" t="s">
         <v>353</v>
@@ -4825,7 +4826,7 @@
         <v>353</v>
       </c>
       <c r="N65" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.3">
@@ -4845,7 +4846,7 @@
         <v>25</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="H66" s="2" t="s">
         <v>353</v>
@@ -4857,7 +4858,7 @@
         <v>2</v>
       </c>
       <c r="K66" s="2" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="L66" s="2" t="s">
         <v>353</v>
@@ -4866,7 +4867,7 @@
         <v>353</v>
       </c>
       <c r="N66" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.3">
@@ -4886,7 +4887,7 @@
         <v>35</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="H67" s="2" t="s">
         <v>353</v>
@@ -4898,7 +4899,7 @@
         <v>3</v>
       </c>
       <c r="K67" s="3" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="L67" s="2" t="s">
         <v>353</v>
@@ -4907,7 +4908,7 @@
         <v>354</v>
       </c>
       <c r="N67" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.3">
@@ -4927,7 +4928,7 @@
         <v>44</v>
       </c>
       <c r="G68" s="2" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="H68" s="2" t="s">
         <v>353</v>
@@ -4939,7 +4940,7 @@
         <v>4</v>
       </c>
       <c r="K68" s="3" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="L68" s="2" t="s">
         <v>353</v>
@@ -4948,7 +4949,7 @@
         <v>354</v>
       </c>
       <c r="N68" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.3">
@@ -4968,7 +4969,7 @@
         <v>43</v>
       </c>
       <c r="G69" s="2" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="H69" s="2" t="s">
         <v>353</v>
@@ -4980,7 +4981,7 @@
         <v>4</v>
       </c>
       <c r="K69" s="3" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="L69" s="2" t="s">
         <v>353</v>
@@ -4989,7 +4990,7 @@
         <v>353</v>
       </c>
       <c r="N69" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.3">
@@ -5009,7 +5010,7 @@
         <v>32</v>
       </c>
       <c r="G70" s="2" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="H70" s="2" t="s">
         <v>353</v>
@@ -5021,7 +5022,7 @@
         <v>3</v>
       </c>
       <c r="K70" s="3" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="L70" s="2" t="s">
         <v>353</v>
@@ -5030,7 +5031,7 @@
         <v>353</v>
       </c>
       <c r="N70" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.3">
@@ -5050,7 +5051,7 @@
         <v>46</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="H71" s="2" t="s">
         <v>353</v>
@@ -5062,7 +5063,7 @@
         <v>5</v>
       </c>
       <c r="K71" s="2" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="L71" s="2" t="s">
         <v>353</v>
@@ -5071,7 +5072,7 @@
         <v>353</v>
       </c>
       <c r="N71" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.3">
@@ -5088,13 +5089,13 @@
         <v>193</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="G72" s="2" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="H72" s="2" t="s">
         <v>353</v>
@@ -5112,7 +5113,7 @@
         <v>354</v>
       </c>
       <c r="N72" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.3">
@@ -5132,10 +5133,10 @@
         <v>188</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="H73" s="2" t="s">
         <v>353</v>
@@ -5147,7 +5148,7 @@
         <v>3</v>
       </c>
       <c r="K73" s="2" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="L73" s="2" t="s">
         <v>353</v>
@@ -5156,7 +5157,7 @@
         <v>354</v>
       </c>
       <c r="N73" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.3">
@@ -5176,7 +5177,7 @@
         <v>189</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="H74" s="2" t="s">
         <v>353</v>
@@ -5194,10 +5195,10 @@
         <v>354</v>
       </c>
       <c r="N74" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="R74" s="2" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.3">
@@ -5229,10 +5230,10 @@
         <v>354</v>
       </c>
       <c r="N75" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="R75" s="2" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.3">
@@ -5249,7 +5250,7 @@
         <v>191</v>
       </c>
       <c r="F76" s="2" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="H76" s="2" t="s">
         <v>353</v>
@@ -5267,7 +5268,7 @@
         <v>354</v>
       </c>
       <c r="N76" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U76" s="2" t="s">
         <v>186</v>
@@ -5290,10 +5291,10 @@
         <v>49</v>
       </c>
       <c r="F77" s="2" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="G77" s="2" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="H77" s="2" t="s">
         <v>353</v>
@@ -5305,7 +5306,7 @@
         <v>4</v>
       </c>
       <c r="K77" s="3" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="L77" s="2" t="s">
         <v>353</v>
@@ -5314,7 +5315,7 @@
         <v>354</v>
       </c>
       <c r="N77" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.3">
@@ -5334,10 +5335,10 @@
         <v>48</v>
       </c>
       <c r="F78" s="2" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="G78" s="2" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="H78" s="2" t="s">
         <v>353</v>
@@ -5349,7 +5350,7 @@
         <v>5</v>
       </c>
       <c r="K78" s="3" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="L78" s="2" t="s">
         <v>353</v>
@@ -5358,7 +5359,7 @@
         <v>354</v>
       </c>
       <c r="N78" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.3">
@@ -5375,7 +5376,7 @@
         <v>139</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H79" s="2" t="s">
         <v>353</v>
@@ -5387,7 +5388,7 @@
         <v>6</v>
       </c>
       <c r="K79" s="2" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="L79" s="2" t="s">
         <v>353</v>
@@ -5396,10 +5397,10 @@
         <v>354</v>
       </c>
       <c r="N79" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="R79" s="2" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.3">
@@ -5434,7 +5435,7 @@
         <v>354</v>
       </c>
       <c r="N80" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U80" s="2" t="s">
         <v>164</v>
@@ -5463,7 +5464,7 @@
         <v>4</v>
       </c>
       <c r="K81" s="3" t="s">
-        <v>606</v>
+        <v>603</v>
       </c>
       <c r="L81" s="3" t="s">
         <v>353</v>
@@ -5472,7 +5473,7 @@
         <v>354</v>
       </c>
       <c r="N81" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="82" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
@@ -5489,7 +5490,7 @@
         <v>150</v>
       </c>
       <c r="F82" s="2" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="H82" s="2" t="s">
         <v>353</v>
@@ -5501,7 +5502,7 @@
         <v>4</v>
       </c>
       <c r="K82" s="3" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="L82" s="2" t="s">
         <v>353</v>
@@ -5510,7 +5511,7 @@
         <v>354</v>
       </c>
       <c r="N82" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="83" spans="1:21" ht="115.2" hidden="1" x14ac:dyDescent="0.3">
@@ -5536,7 +5537,7 @@
         <v>354</v>
       </c>
       <c r="N83" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="84" spans="1:21" ht="115.2" x14ac:dyDescent="0.3">
@@ -5574,10 +5575,10 @@
         <v>354</v>
       </c>
       <c r="N84" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="R84" s="2" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
     </row>
     <row r="85" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
@@ -5609,7 +5610,7 @@
         <v>354</v>
       </c>
       <c r="N85" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="86" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
@@ -5641,7 +5642,7 @@
         <v>354</v>
       </c>
       <c r="N86" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="87" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
@@ -5673,7 +5674,7 @@
         <v>354</v>
       </c>
       <c r="N87" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="88" spans="1:21" x14ac:dyDescent="0.3">
@@ -5687,10 +5688,10 @@
         <v>193</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="H88" s="2" t="s">
         <v>353</v>
@@ -5702,7 +5703,7 @@
         <v>1</v>
       </c>
       <c r="K88" s="3" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="L88" s="2" t="s">
         <v>353</v>
@@ -5711,7 +5712,7 @@
         <v>354</v>
       </c>
       <c r="N88" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="89" spans="1:21" x14ac:dyDescent="0.3">
@@ -5725,7 +5726,7 @@
         <v>193</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="H89" s="2" t="s">
         <v>353</v>
@@ -5737,7 +5738,7 @@
         <v>1</v>
       </c>
       <c r="K89" s="2" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="L89" s="2" t="s">
         <v>353</v>
@@ -5746,7 +5747,7 @@
         <v>354</v>
       </c>
       <c r="N89" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="90" spans="1:21" x14ac:dyDescent="0.3">
@@ -5760,10 +5761,10 @@
         <v>193</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="F90" s="2" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="H90" s="2" t="s">
         <v>353</v>
@@ -5781,12 +5782,12 @@
         <v>354</v>
       </c>
       <c r="N90" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="91" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A91" s="2" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B91" s="2" t="s">
         <v>2</v>
@@ -5795,22 +5796,22 @@
         <v>193</v>
       </c>
       <c r="E91" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="F91" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="H91" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="I91" s="2" t="s">
         <v>382</v>
       </c>
-      <c r="F91" s="2" t="s">
-        <v>495</v>
-      </c>
-      <c r="H91" s="2" t="s">
-        <v>353</v>
-      </c>
-      <c r="I91" s="2" t="s">
-        <v>384</v>
-      </c>
       <c r="J91" s="2" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="K91" s="2" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="L91" s="2" t="s">
         <v>353</v>
@@ -5819,7 +5820,7 @@
         <v>354</v>
       </c>
       <c r="N91" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="92" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
@@ -5836,7 +5837,7 @@
         <v>353</v>
       </c>
       <c r="K92" s="2" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="L92" s="2" t="s">
         <v>354</v>
@@ -5845,7 +5846,7 @@
         <v>354</v>
       </c>
       <c r="N92" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="93" spans="1:21" x14ac:dyDescent="0.3">
@@ -5865,7 +5866,7 @@
         <v>59</v>
       </c>
       <c r="F93" s="2" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="H93" s="2" t="s">
         <v>353</v>
@@ -5877,7 +5878,7 @@
         <v>6</v>
       </c>
       <c r="K93" s="2" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="L93" s="2" t="s">
         <v>353</v>
@@ -5886,7 +5887,7 @@
         <v>353</v>
       </c>
       <c r="N93" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="94" spans="1:21" x14ac:dyDescent="0.3">
@@ -5906,10 +5907,10 @@
         <v>24</v>
       </c>
       <c r="F94" s="2" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="G94" s="2" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="H94" s="2" t="s">
         <v>353</v>
@@ -5921,7 +5922,7 @@
         <v>2</v>
       </c>
       <c r="K94" s="2" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="L94" s="2" t="s">
         <v>353</v>
@@ -5930,7 +5931,7 @@
         <v>353</v>
       </c>
       <c r="N94" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U94" s="2" t="s">
         <v>159</v>
@@ -5953,7 +5954,7 @@
         <v>45</v>
       </c>
       <c r="G95" s="2" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="H95" s="2" t="s">
         <v>353</v>
@@ -5965,7 +5966,7 @@
         <v>5</v>
       </c>
       <c r="K95" s="2" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="L95" s="2" t="s">
         <v>353</v>
@@ -5974,7 +5975,7 @@
         <v>353</v>
       </c>
       <c r="N95" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="96" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
@@ -6000,7 +6001,7 @@
         <v>3</v>
       </c>
       <c r="K96" s="2" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="L96" s="2" t="s">
         <v>354</v>
@@ -6009,7 +6010,7 @@
         <v>353</v>
       </c>
       <c r="N96" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="97" spans="1:21" ht="129.6" x14ac:dyDescent="0.3">
@@ -6026,13 +6027,13 @@
         <v>353</v>
       </c>
       <c r="I97" s="2" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="J97" s="2" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="K97" s="3" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="L97" s="3" t="s">
         <v>353</v>
@@ -6041,7 +6042,7 @@
         <v>354</v>
       </c>
       <c r="N97" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="98" spans="1:21" x14ac:dyDescent="0.3">
@@ -6073,10 +6074,10 @@
         <v>354</v>
       </c>
       <c r="N98" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="R98" s="2" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
     </row>
     <row r="99" spans="1:21" x14ac:dyDescent="0.3">
@@ -6090,7 +6091,7 @@
         <v>195</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="F99" s="2" t="s">
         <v>142</v>
@@ -6105,7 +6106,7 @@
         <v>2</v>
       </c>
       <c r="K99" s="2" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="L99" s="2" t="s">
         <v>353</v>
@@ -6114,10 +6115,10 @@
         <v>354</v>
       </c>
       <c r="N99" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="P99" s="2" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
     </row>
     <row r="100" spans="1:21" x14ac:dyDescent="0.3">
@@ -6134,7 +6135,7 @@
         <v>153</v>
       </c>
       <c r="F100" s="2" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="H100" s="2" t="s">
         <v>353</v>
@@ -6146,7 +6147,7 @@
         <v>6</v>
       </c>
       <c r="K100" s="2" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="L100" s="2" t="s">
         <v>353</v>
@@ -6155,7 +6156,7 @@
         <v>353</v>
       </c>
       <c r="N100" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="101" spans="1:21" x14ac:dyDescent="0.3">
@@ -6181,7 +6182,7 @@
         <v>5</v>
       </c>
       <c r="K101" s="3" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="L101" s="2" t="s">
         <v>353</v>
@@ -6190,7 +6191,7 @@
         <v>354</v>
       </c>
       <c r="N101" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="102" spans="1:21" x14ac:dyDescent="0.3">
@@ -6216,7 +6217,7 @@
         <v>4</v>
       </c>
       <c r="K102" s="2" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="L102" s="2" t="s">
         <v>353</v>
@@ -6225,7 +6226,7 @@
         <v>354</v>
       </c>
       <c r="N102" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="103" spans="1:21" x14ac:dyDescent="0.3">
@@ -6263,7 +6264,7 @@
         <v>354</v>
       </c>
       <c r="N103" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="104" spans="1:21" x14ac:dyDescent="0.3">
@@ -6277,10 +6278,10 @@
         <v>195</v>
       </c>
       <c r="E104" s="2" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="F104" s="2" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="H104" s="2" t="s">
         <v>353</v>
@@ -6298,13 +6299,13 @@
         <v>354</v>
       </c>
       <c r="N104" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="P104" s="2" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="R104" s="2" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="U104" s="2" t="s">
         <v>167</v>
@@ -6333,7 +6334,7 @@
         <v>354</v>
       </c>
       <c r="N105" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U105" s="2" t="s">
         <v>357</v>
@@ -6368,7 +6369,7 @@
         <v>4</v>
       </c>
       <c r="K106" s="3" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="L106" s="2" t="s">
         <v>353</v>
@@ -6377,7 +6378,7 @@
         <v>354</v>
       </c>
       <c r="N106" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U106" s="2" t="s">
         <v>162</v>
@@ -6409,7 +6410,7 @@
         <v>5</v>
       </c>
       <c r="K107" s="3" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="L107" s="2" t="s">
         <v>353</v>
@@ -6418,10 +6419,10 @@
         <v>354</v>
       </c>
       <c r="N107" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U107" s="2" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
     </row>
     <row r="108" spans="1:21" x14ac:dyDescent="0.3">
@@ -6450,7 +6451,7 @@
         <v>6</v>
       </c>
       <c r="K108" s="2" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="L108" s="2" t="s">
         <v>353</v>
@@ -6459,10 +6460,10 @@
         <v>353</v>
       </c>
       <c r="N108" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="P108" s="2" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="U108" s="2" t="s">
         <v>162</v>
@@ -6491,7 +6492,7 @@
         <v>6</v>
       </c>
       <c r="K109" s="3" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="L109" s="2" t="s">
         <v>353</v>
@@ -6500,7 +6501,7 @@
         <v>354</v>
       </c>
       <c r="N109" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="110" spans="1:21" x14ac:dyDescent="0.3">
@@ -6526,7 +6527,7 @@
         <v>7</v>
       </c>
       <c r="K110" s="9" t="s">
-        <v>604</v>
+        <v>601</v>
       </c>
       <c r="L110" s="10" t="s">
         <v>353</v>
@@ -6535,10 +6536,10 @@
         <v>354</v>
       </c>
       <c r="N110" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="R110" s="2" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
     </row>
     <row r="111" spans="1:21" x14ac:dyDescent="0.3">
@@ -6564,7 +6565,7 @@
         <v>4</v>
       </c>
       <c r="K111" s="2" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="L111" s="2" t="s">
         <v>353</v>
@@ -6573,7 +6574,7 @@
         <v>353</v>
       </c>
       <c r="N111" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="112" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -6600,7 +6601,7 @@
         <v>3</v>
       </c>
       <c r="K112" s="2" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="L112" s="2" t="s">
         <v>353</v>
@@ -6609,10 +6610,10 @@
         <v>354</v>
       </c>
       <c r="N112" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U112" s="3" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
     </row>
     <row r="113" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
@@ -6647,7 +6648,7 @@
         <v>354</v>
       </c>
       <c r="N113" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="114" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
@@ -6661,7 +6662,7 @@
         <v>193</v>
       </c>
       <c r="E114" s="2" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="H114" s="2" t="s">
         <v>353</v>
@@ -6673,7 +6674,7 @@
         <v>1</v>
       </c>
       <c r="K114" s="3" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="L114" s="2" t="s">
         <v>354</v>
@@ -6682,7 +6683,7 @@
         <v>353</v>
       </c>
       <c r="N114" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="115" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
@@ -6708,7 +6709,7 @@
         <v>1</v>
       </c>
       <c r="K115" s="3" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
       <c r="L115" s="3" t="s">
         <v>353</v>
@@ -6717,10 +6718,10 @@
         <v>354</v>
       </c>
       <c r="N115" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U115" s="2" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
     </row>
     <row r="116" spans="1:21" x14ac:dyDescent="0.3">
@@ -6740,7 +6741,7 @@
         <v>79</v>
       </c>
       <c r="G116" s="2" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="H116" s="2" t="s">
         <v>353</v>
@@ -6752,7 +6753,7 @@
         <v>3</v>
       </c>
       <c r="K116" s="2" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="L116" s="2" t="s">
         <v>353</v>
@@ -6761,7 +6762,7 @@
         <v>354</v>
       </c>
       <c r="N116" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="117" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
@@ -6789,7 +6790,7 @@
         <v>354</v>
       </c>
       <c r="N117" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="118" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
@@ -6814,7 +6815,7 @@
         <v>354</v>
       </c>
       <c r="N118" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="119" spans="1:21" x14ac:dyDescent="0.3">
@@ -6849,7 +6850,7 @@
         <v>354</v>
       </c>
       <c r="N119" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U119" s="2" t="s">
         <v>185</v>
@@ -6872,7 +6873,7 @@
         <v>40</v>
       </c>
       <c r="G120" s="2" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="H120" s="2" t="s">
         <v>353</v>
@@ -6884,7 +6885,7 @@
         <v>3</v>
       </c>
       <c r="K120" s="3" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="L120" s="2" t="s">
         <v>353</v>
@@ -6893,7 +6894,7 @@
         <v>354</v>
       </c>
       <c r="N120" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="121" spans="1:21" x14ac:dyDescent="0.3">
@@ -6919,7 +6920,7 @@
         <v>4</v>
       </c>
       <c r="K121" s="2" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="L121" s="2" t="s">
         <v>353</v>
@@ -6928,7 +6929,7 @@
         <v>354</v>
       </c>
       <c r="N121" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="122" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
@@ -6954,7 +6955,7 @@
         <v>3</v>
       </c>
       <c r="K122" s="2" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="L122" s="2" t="s">
         <v>354</v>
@@ -6963,7 +6964,7 @@
         <v>353</v>
       </c>
       <c r="N122" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="123" spans="1:21" x14ac:dyDescent="0.3">
@@ -6998,7 +6999,7 @@
         <v>353</v>
       </c>
       <c r="N123" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="124" spans="1:21" x14ac:dyDescent="0.3">
@@ -7018,10 +7019,10 @@
         <v>71</v>
       </c>
       <c r="F124" s="2" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="G124" s="2" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="H124" s="2" t="s">
         <v>353</v>
@@ -7033,7 +7034,7 @@
         <v>4</v>
       </c>
       <c r="K124" s="3" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="L124" s="2" t="s">
         <v>353</v>
@@ -7042,7 +7043,7 @@
         <v>354</v>
       </c>
       <c r="N124" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="125" spans="1:21" x14ac:dyDescent="0.3">
@@ -7062,7 +7063,7 @@
         <v>73</v>
       </c>
       <c r="G125" s="2" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="H125" s="2" t="s">
         <v>353</v>
@@ -7074,7 +7075,7 @@
         <v>5</v>
       </c>
       <c r="K125" s="2" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="L125" s="2" t="s">
         <v>353</v>
@@ -7083,10 +7084,10 @@
         <v>354</v>
       </c>
       <c r="N125" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U125" s="2" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="126" spans="1:21" x14ac:dyDescent="0.3">
@@ -7106,7 +7107,7 @@
         <v>75</v>
       </c>
       <c r="G126" s="2" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="H126" s="2" t="s">
         <v>353</v>
@@ -7118,7 +7119,7 @@
         <v>6</v>
       </c>
       <c r="K126" s="2" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="L126" s="2" t="s">
         <v>353</v>
@@ -7127,7 +7128,7 @@
         <v>353</v>
       </c>
       <c r="N126" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="127" spans="1:21" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
@@ -7159,7 +7160,7 @@
         <v>354</v>
       </c>
       <c r="N127" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U127" s="2" t="s">
         <v>184</v>
@@ -7188,7 +7189,7 @@
         <v>6</v>
       </c>
       <c r="K128" s="2" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="L128" s="2" t="s">
         <v>353</v>
@@ -7197,7 +7198,7 @@
         <v>354</v>
       </c>
       <c r="N128" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="129" spans="1:21" x14ac:dyDescent="0.3">
@@ -7229,7 +7230,7 @@
         <v>354</v>
       </c>
       <c r="N129" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="130" spans="1:21" x14ac:dyDescent="0.3">
@@ -7249,7 +7250,7 @@
         <v>80</v>
       </c>
       <c r="G130" s="2" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="H130" s="2" t="s">
         <v>353</v>
@@ -7261,7 +7262,7 @@
         <v>4</v>
       </c>
       <c r="K130" s="2" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="L130" s="2" t="s">
         <v>353</v>
@@ -7270,7 +7271,7 @@
         <v>354</v>
       </c>
       <c r="N130" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="131" spans="1:21" x14ac:dyDescent="0.3">
@@ -7290,7 +7291,7 @@
         <v>81</v>
       </c>
       <c r="G131" s="2" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="H131" s="2" t="s">
         <v>353</v>
@@ -7302,7 +7303,7 @@
         <v>5</v>
       </c>
       <c r="K131" s="2" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="L131" s="2" t="s">
         <v>353</v>
@@ -7311,7 +7312,7 @@
         <v>354</v>
       </c>
       <c r="N131" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="132" spans="1:21" x14ac:dyDescent="0.3">
@@ -7331,10 +7332,10 @@
         <v>82</v>
       </c>
       <c r="F132" s="2" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="G132" s="2" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="H132" s="2" t="s">
         <v>353</v>
@@ -7346,7 +7347,7 @@
         <v>6</v>
       </c>
       <c r="K132" s="2" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="L132" s="2" t="s">
         <v>353</v>
@@ -7355,10 +7356,10 @@
         <v>354</v>
       </c>
       <c r="N132" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="P132" s="2" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
     </row>
     <row r="133" spans="1:21" x14ac:dyDescent="0.3">
@@ -7375,7 +7376,7 @@
         <v>105</v>
       </c>
       <c r="F133" s="10" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="G133" s="10"/>
       <c r="H133" s="2" t="s">
@@ -7388,7 +7389,7 @@
         <v>6</v>
       </c>
       <c r="K133" s="3" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="L133" s="2" t="s">
         <v>353</v>
@@ -7397,7 +7398,7 @@
         <v>354</v>
       </c>
       <c r="N133" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="134" spans="1:21" x14ac:dyDescent="0.3">
@@ -7418,7 +7419,7 @@
       </c>
       <c r="F134" s="10"/>
       <c r="G134" s="10" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="H134" s="2" t="s">
         <v>353</v>
@@ -7436,7 +7437,7 @@
         <v>354</v>
       </c>
       <c r="N134" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="135" spans="1:21" x14ac:dyDescent="0.3">
@@ -7459,7 +7460,7 @@
         <v>204</v>
       </c>
       <c r="G135" s="10" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="H135" s="2" t="s">
         <v>353</v>
@@ -7471,7 +7472,7 @@
         <v>3</v>
       </c>
       <c r="K135" s="3" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="L135" s="2" t="s">
         <v>353</v>
@@ -7480,7 +7481,7 @@
         <v>354</v>
       </c>
       <c r="N135" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="136" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
@@ -7500,7 +7501,7 @@
         <v>41</v>
       </c>
       <c r="G136" s="2" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="H136" s="2" t="s">
         <v>353</v>
@@ -7518,7 +7519,7 @@
         <v>354</v>
       </c>
       <c r="N136" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="137" spans="1:21" x14ac:dyDescent="0.3">
@@ -7544,7 +7545,7 @@
         <v>4</v>
       </c>
       <c r="K137" s="2" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="L137" s="2" t="s">
         <v>353</v>
@@ -7553,7 +7554,7 @@
         <v>354</v>
       </c>
       <c r="N137" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="138" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
@@ -7582,10 +7583,10 @@
         <v>354</v>
       </c>
       <c r="N138" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U138" s="2" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
     </row>
     <row r="139" spans="1:21" ht="72" x14ac:dyDescent="0.3">
@@ -7611,7 +7612,7 @@
         <v>7</v>
       </c>
       <c r="K139" s="3" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="L139" s="2" t="s">
         <v>353</v>
@@ -7620,10 +7621,10 @@
         <v>354</v>
       </c>
       <c r="N139" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="R139" s="2" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
     </row>
     <row r="140" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
@@ -7640,7 +7641,7 @@
         <v>6</v>
       </c>
       <c r="F140" s="2" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="H140" s="2" t="s">
         <v>353</v>
@@ -7652,7 +7653,7 @@
         <v>1</v>
       </c>
       <c r="K140" s="3" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
       <c r="L140" s="2" t="s">
         <v>353</v>
@@ -7661,7 +7662,7 @@
         <v>353</v>
       </c>
       <c r="N140" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="141" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
@@ -7696,7 +7697,7 @@
         <v>354</v>
       </c>
       <c r="N141" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U141" s="2" t="s">
         <v>196</v>
@@ -7713,7 +7714,7 @@
         <v>194</v>
       </c>
       <c r="E142" s="2" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="H142" s="2" t="s">
         <v>353</v>
@@ -7722,7 +7723,7 @@
         <v>361</v>
       </c>
       <c r="J142" s="2" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="L142" s="2" t="s">
         <v>354</v>
@@ -7731,7 +7732,7 @@
         <v>354</v>
       </c>
       <c r="N142" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U142" s="12" t="s">
         <v>362</v>
@@ -7739,25 +7740,25 @@
     </row>
     <row r="143" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A143" s="2" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="B143" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="E143" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="H143" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="I143" s="2" t="s">
         <v>396</v>
       </c>
-      <c r="E143" s="2" t="s">
-        <v>397</v>
-      </c>
-      <c r="H143" s="2" t="s">
-        <v>353</v>
-      </c>
-      <c r="I143" s="2" t="s">
-        <v>398</v>
-      </c>
       <c r="J143" s="2" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="K143" s="2" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="L143" s="2" t="s">
         <v>353</v>
@@ -7766,62 +7767,62 @@
         <v>354</v>
       </c>
       <c r="N143" s="2" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="U143" s="2" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="144" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A144" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="B144" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="E144" s="2" t="s">
         <v>391</v>
       </c>
-      <c r="B144" s="2" t="s">
-        <v>396</v>
-      </c>
-      <c r="E144" s="2" t="s">
+      <c r="H144" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="I144" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="K144" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="L144" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="M144" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="N144" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="U144" s="2" t="s">
         <v>393</v>
-      </c>
-      <c r="H144" s="2" t="s">
-        <v>353</v>
-      </c>
-      <c r="I144" s="2" t="s">
-        <v>394</v>
-      </c>
-      <c r="K144" s="2" t="s">
-        <v>448</v>
-      </c>
-      <c r="L144" s="2" t="s">
-        <v>353</v>
-      </c>
-      <c r="M144" s="2" t="s">
-        <v>354</v>
-      </c>
-      <c r="N144" s="2" t="s">
-        <v>442</v>
-      </c>
-      <c r="U144" s="2" t="s">
-        <v>395</v>
       </c>
     </row>
     <row r="145" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A145" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="B145" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="E145" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="H145" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="I145" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="B145" s="2" t="s">
-        <v>396</v>
-      </c>
-      <c r="E145" s="2" t="s">
-        <v>399</v>
-      </c>
-      <c r="H145" s="2" t="s">
-        <v>353</v>
-      </c>
-      <c r="I145" s="2" t="s">
-        <v>394</v>
-      </c>
       <c r="K145" s="2" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="L145" s="2" t="s">
         <v>353</v>
@@ -7830,33 +7831,33 @@
         <v>354</v>
       </c>
       <c r="N145" s="2" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="U145" s="2" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="146" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A146" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="B146" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="E146" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="H146" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="I146" s="2" t="s">
         <v>400</v>
       </c>
-      <c r="B146" s="2" t="s">
-        <v>396</v>
-      </c>
-      <c r="E146" s="2" t="s">
-        <v>454</v>
-      </c>
-      <c r="H146" s="2" t="s">
-        <v>353</v>
-      </c>
-      <c r="I146" s="2" t="s">
-        <v>402</v>
-      </c>
       <c r="J146" s="2" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="K146" s="2" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="L146" s="2" t="s">
         <v>353</v>
@@ -7865,33 +7866,33 @@
         <v>354</v>
       </c>
       <c r="N146" s="2" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="U146" s="2" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="147" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A147" s="2" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="E147" s="2" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="H147" s="2" t="s">
         <v>353</v>
       </c>
       <c r="I147" s="2" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="J147" s="2" t="s">
         <v>363</v>
       </c>
       <c r="K147" s="2" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="L147" s="2" t="s">
         <v>353</v>
@@ -7900,36 +7901,36 @@
         <v>354</v>
       </c>
       <c r="N147" s="2" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
     </row>
     <row r="148" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A148" s="2" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="B148" s="2" t="s">
         <v>83</v>
       </c>
       <c r="D148" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="E148" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="F148" s="2" t="s">
+        <v>535</v>
+      </c>
+      <c r="H148" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="I148" s="2" t="s">
         <v>408</v>
       </c>
-      <c r="E148" s="2" t="s">
+      <c r="J148" s="2" t="s">
         <v>409</v>
       </c>
-      <c r="F148" s="2" t="s">
-        <v>537</v>
-      </c>
-      <c r="H148" s="2" t="s">
-        <v>353</v>
-      </c>
-      <c r="I148" s="2" t="s">
-        <v>410</v>
-      </c>
-      <c r="J148" s="2" t="s">
-        <v>411</v>
-      </c>
       <c r="K148" s="2" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="L148" s="2" t="s">
         <v>353</v>
@@ -7938,28 +7939,28 @@
         <v>354</v>
       </c>
       <c r="N148" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="149" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A149" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="B149" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="E149" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="H149" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="I149" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="K149" s="2" t="s">
         <v>443</v>
       </c>
-      <c r="B149" s="2" t="s">
-        <v>396</v>
-      </c>
-      <c r="E149" s="2" t="s">
-        <v>376</v>
-      </c>
-      <c r="H149" s="2" t="s">
-        <v>354</v>
-      </c>
-      <c r="I149" s="2" t="s">
-        <v>444</v>
-      </c>
-      <c r="K149" s="2" t="s">
-        <v>445</v>
-      </c>
       <c r="L149" s="2" t="s">
         <v>354</v>
       </c>
@@ -7967,33 +7968,33 @@
         <v>353</v>
       </c>
       <c r="N149" s="2" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="U149" s="2" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="150" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A150" s="2" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="E150" s="2" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="H150" s="2" t="s">
         <v>353</v>
       </c>
       <c r="I150" s="2" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="J150" s="2" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="K150" s="2" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="L150" s="2" t="s">
         <v>353</v>
@@ -8002,30 +8003,30 @@
         <v>354</v>
       </c>
       <c r="N150" s="2" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
     </row>
     <row r="151" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A151" s="2" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="E151" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="H151" s="2" t="s">
         <v>353</v>
       </c>
       <c r="I151" s="2" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="J151" s="2" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="K151" s="2" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="L151" s="2" t="s">
         <v>353</v>
@@ -8034,30 +8035,30 @@
         <v>354</v>
       </c>
       <c r="N151" s="2" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
     </row>
     <row r="152" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A152" s="2" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="E152" s="2" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="H152" s="2" t="s">
         <v>353</v>
       </c>
       <c r="I152" s="2" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="J152" s="2" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="K152" s="2" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="L152" s="2" t="s">
         <v>353</v>
@@ -8066,30 +8067,30 @@
         <v>354</v>
       </c>
       <c r="N152" s="2" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
     </row>
     <row r="153" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A153" s="2" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="E153" s="2" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="H153" s="2" t="s">
         <v>353</v>
       </c>
       <c r="I153" s="2" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="J153" s="2" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="K153" s="2" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="L153" s="2" t="s">
         <v>353</v>
@@ -8098,30 +8099,30 @@
         <v>354</v>
       </c>
       <c r="N153" s="2" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="R153" s="2" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
     </row>
     <row r="154" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A154" s="2" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="E154" s="2" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="H154" s="2" t="s">
         <v>353</v>
       </c>
       <c r="I154" s="2" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="K154" s="2" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="L154" s="2" t="s">
         <v>353</v>
@@ -8130,24 +8131,24 @@
         <v>354</v>
       </c>
       <c r="N154" s="2" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
     </row>
     <row r="155" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A155" s="2" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="E155" s="2" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="H155" s="2" t="s">
         <v>353</v>
       </c>
       <c r="K155" s="2" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="L155" s="2" t="s">
         <v>353</v>
@@ -8156,12 +8157,12 @@
         <v>354</v>
       </c>
       <c r="N155" s="2" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
     </row>
     <row r="156" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A156" s="2" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="B156" s="2" t="s">
         <v>125</v>
@@ -8173,19 +8174,19 @@
         <v>139</v>
       </c>
       <c r="F156" s="2" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H156" s="2" t="s">
         <v>353</v>
       </c>
       <c r="I156" s="2" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="J156" s="2">
         <v>6</v>
       </c>
       <c r="K156" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="L156" s="2" t="s">
         <v>353</v>
@@ -8194,13 +8195,13 @@
         <v>354</v>
       </c>
       <c r="N156" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="R156" s="2" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
       <c r="U156" s="2" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
SAS confidence, table generation
</commit_message>
<xml_diff>
--- a/src/sastadev/data/methods/TARSP_Index_Current.xlsx
+++ b/src/sastadev/data/methods/TARSP_Index_Current.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\jodijk\myprograms\python\sastacode\mysastadev\src\sastadev\data\methods\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C490BD60-AD31-49E5-90D6-F70FAA494A41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4153D081-55A2-4EF0-BD09-918A2FFAA5B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1882,9 +1882,6 @@
     <t>//node[@lemma="alles"  or @lemma="niets" or @lemma="niks" or %zelfst_wat% or (@lemma="u" and not(../node[%dankje_VU%])) or @lemma="ons"  or @lemma="zelf"]</t>
   </si>
   <si>
-    <t xml:space="preserve">dir </t>
-  </si>
-  <si>
     <t>//node[(@pt="n" or @pt="tw") and %realwordnode% and @lemma!="kijk" and %thisistheonlyrealword%]</t>
   </si>
   <si>
@@ -1917,6 +1914,9 @@
   </si>
   <si>
     <t>bx</t>
+  </si>
+  <si>
+    <t>tarsp2017,tarspauris</t>
   </si>
 </sst>
 </file>
@@ -2724,7 +2724,7 @@
         <v>6</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="L9" s="2" t="s">
         <v>352</v>
@@ -3273,7 +3273,7 @@
         <v>2</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="L24" s="2" t="s">
         <v>352</v>
@@ -3381,7 +3381,7 @@
         <v>4</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="L27" s="2" t="s">
         <v>352</v>
@@ -3416,7 +3416,7 @@
         <v>5</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="L28" s="2" t="s">
         <v>352</v>
@@ -3717,7 +3717,7 @@
         <v>5</v>
       </c>
       <c r="K36" s="3" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="L36" s="3" t="s">
         <v>352</v>
@@ -3951,7 +3951,7 @@
         <v>2</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="L42" s="2" t="s">
         <v>352</v>
@@ -5460,7 +5460,7 @@
         <v>4</v>
       </c>
       <c r="K81" s="3" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="L81" s="3" t="s">
         <v>352</v>
@@ -6916,7 +6916,7 @@
         <v>4</v>
       </c>
       <c r="K121" s="2" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="L121" s="2" t="s">
         <v>352</v>
@@ -7649,7 +7649,7 @@
         <v>1</v>
       </c>
       <c r="K140" s="3" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="L140" s="2" t="s">
         <v>352</v>
@@ -7684,7 +7684,7 @@
         <v>4</v>
       </c>
       <c r="K141" s="3" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="L141" s="3" t="s">
         <v>352</v>
@@ -8194,7 +8194,7 @@
         <v>437</v>
       </c>
       <c r="R156" s="2" t="s">
-        <v>601</v>
+        <v>611</v>
       </c>
       <c r="U156" s="2" t="s">
         <v>588</v>

</xml_diff>

<commit_message>
initial ov2; sort_order_functions; update of resultsbyutterance
</commit_message>
<xml_diff>
--- a/src/sastadev/data/methods/TARSP_Index_Current.xlsx
+++ b/src/sastadev/data/methods/TARSP_Index_Current.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\jodijk\myprograms\python\sastacode\mysastadev\src\sastadev\data\methods\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82135B13-C850-452C-96D7-C7CD0A11BD12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECD5D6FA-6ED0-47A6-B6D9-229F7178F3B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1843,9 +1843,6 @@
     <t>taalmaat is veranderd in 2017; vgl T085</t>
   </si>
   <si>
-    <t>//node[node[(@lemma="een" or @lemma="'n") and @pt="lid"] and node[(@pt="n" or (@pt="adj" and @positie="nom")) and @rel="hd"] and count(node)=2 ]</t>
-  </si>
-  <si>
     <t>bbx</t>
   </si>
   <si>
@@ -1917,6 +1914,9 @@
   </si>
   <si>
     <t>//node[%AVn%]</t>
+  </si>
+  <si>
+    <t>//node[%Tarsp_een%]</t>
   </si>
 </sst>
 </file>
@@ -2334,6 +2334,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:V156"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2417,7 +2418,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>212</v>
       </c>
@@ -2464,7 +2465,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>213</v>
       </c>
@@ -2505,7 +2506,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>214</v>
       </c>
@@ -2546,7 +2547,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>215</v>
       </c>
@@ -2584,7 +2585,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>216</v>
       </c>
@@ -2607,7 +2608,7 @@
         <v>1</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>352</v>
@@ -2625,7 +2626,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>217</v>
       </c>
@@ -2660,7 +2661,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="8" spans="1:22" ht="115.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:22" ht="115.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>218</v>
       </c>
@@ -2698,7 +2699,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>219</v>
       </c>
@@ -2724,7 +2725,7 @@
         <v>6</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="L9" s="2" t="s">
         <v>352</v>
@@ -2739,7 +2740,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="10" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:22" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>220</v>
       </c>
@@ -2774,7 +2775,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>221</v>
       </c>
@@ -2809,7 +2810,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>222</v>
       </c>
@@ -2838,7 +2839,7 @@
         <v>3</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="L12" s="2" t="s">
         <v>352</v>
@@ -2850,7 +2851,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>223</v>
       </c>
@@ -2873,7 +2874,7 @@
         <v>5</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="L13" s="3" t="s">
         <v>352</v>
@@ -2885,7 +2886,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>224</v>
       </c>
@@ -2923,7 +2924,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>225</v>
       </c>
@@ -2946,7 +2947,7 @@
         <v>4</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="L15" s="2" t="s">
         <v>352</v>
@@ -2958,7 +2959,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>226</v>
       </c>
@@ -2987,7 +2988,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>227</v>
       </c>
@@ -3019,7 +3020,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>228</v>
       </c>
@@ -3060,7 +3061,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>229</v>
       </c>
@@ -3086,7 +3087,7 @@
         <v>1</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="L19" s="2" t="s">
         <v>352</v>
@@ -3098,7 +3099,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>230</v>
       </c>
@@ -3130,7 +3131,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>231</v>
       </c>
@@ -3153,7 +3154,7 @@
         <v>4</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="L21" s="2" t="s">
         <v>352</v>
@@ -3165,7 +3166,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>232</v>
       </c>
@@ -3200,7 +3201,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>233</v>
       </c>
@@ -3273,7 +3274,7 @@
         <v>2</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="L24" s="2" t="s">
         <v>352</v>
@@ -3288,7 +3289,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>235</v>
       </c>
@@ -3320,7 +3321,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="26" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:21" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>236</v>
       </c>
@@ -3358,7 +3359,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="27" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:21" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>237</v>
       </c>
@@ -3381,7 +3382,7 @@
         <v>4</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="L27" s="2" t="s">
         <v>352</v>
@@ -3393,7 +3394,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>238</v>
       </c>
@@ -3416,7 +3417,7 @@
         <v>5</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="L28" s="2" t="s">
         <v>352</v>
@@ -3451,7 +3452,7 @@
         <v>2</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>588</v>
+        <v>611</v>
       </c>
       <c r="L29" s="2" t="s">
         <v>352</v>
@@ -3466,7 +3467,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>240</v>
       </c>
@@ -3504,7 +3505,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>241</v>
       </c>
@@ -3542,7 +3543,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="32" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:21" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>242</v>
       </c>
@@ -3580,7 +3581,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="33" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>243</v>
       </c>
@@ -3624,7 +3625,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>244</v>
       </c>
@@ -3659,7 +3660,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="35" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>245</v>
       </c>
@@ -3694,7 +3695,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="36" spans="1:21" ht="72" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:21" ht="72" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>246</v>
       </c>
@@ -3717,7 +3718,7 @@
         <v>5</v>
       </c>
       <c r="K36" s="3" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="L36" s="3" t="s">
         <v>352</v>
@@ -3729,7 +3730,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="37" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>247</v>
       </c>
@@ -3764,7 +3765,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="38" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>248</v>
       </c>
@@ -3805,7 +3806,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="39" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>249</v>
       </c>
@@ -3846,7 +3847,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="40" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>250</v>
       </c>
@@ -3887,7 +3888,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>251</v>
       </c>
@@ -3951,7 +3952,7 @@
         <v>2</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="L42" s="2" t="s">
         <v>352</v>
@@ -3966,7 +3967,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="43" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:21" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>253</v>
       </c>
@@ -4010,7 +4011,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>254</v>
       </c>
@@ -4033,7 +4034,7 @@
         <v>3</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="L44" s="2" t="s">
         <v>352</v>
@@ -4045,7 +4046,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="45" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:21" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>255</v>
       </c>
@@ -4124,7 +4125,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="47" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:21" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>257</v>
       </c>
@@ -4162,7 +4163,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="48" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:21" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>258</v>
       </c>
@@ -4191,7 +4192,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="49" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>259</v>
       </c>
@@ -4226,7 +4227,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="50" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:21" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>260</v>
       </c>
@@ -4261,7 +4262,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="51" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>261</v>
       </c>
@@ -4334,7 +4335,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="53" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>263</v>
       </c>
@@ -4357,7 +4358,7 @@
         <v>6</v>
       </c>
       <c r="K53" s="2" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="L53" s="2" t="s">
         <v>352</v>
@@ -4369,7 +4370,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="54" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>264</v>
       </c>
@@ -4407,7 +4408,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="55" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>265</v>
       </c>
@@ -4442,7 +4443,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="56" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>266</v>
       </c>
@@ -4477,7 +4478,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="57" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>267</v>
       </c>
@@ -4553,7 +4554,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="59" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>269</v>
       </c>
@@ -4594,7 +4595,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="60" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>270</v>
       </c>
@@ -4635,7 +4636,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="61" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>271</v>
       </c>
@@ -4673,7 +4674,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="62" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>272</v>
       </c>
@@ -4711,7 +4712,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="63" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>273</v>
       </c>
@@ -4749,7 +4750,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="64" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>274</v>
       </c>
@@ -4866,7 +4867,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="67" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>277</v>
       </c>
@@ -4907,7 +4908,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="68" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>278</v>
       </c>
@@ -4948,7 +4949,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="69" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>279</v>
       </c>
@@ -4989,7 +4990,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="70" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>280</v>
       </c>
@@ -5030,7 +5031,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="71" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>281</v>
       </c>
@@ -5112,7 +5113,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="73" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>283</v>
       </c>
@@ -5156,7 +5157,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="74" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
         <v>284</v>
       </c>
@@ -5197,7 +5198,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="75" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
         <v>285</v>
       </c>
@@ -5232,7 +5233,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="76" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
         <v>286</v>
       </c>
@@ -5270,7 +5271,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="77" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
         <v>287</v>
       </c>
@@ -5314,7 +5315,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="78" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
         <v>288</v>
       </c>
@@ -5358,7 +5359,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="79" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
         <v>289</v>
       </c>
@@ -5384,7 +5385,7 @@
         <v>6</v>
       </c>
       <c r="K79" s="2" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="L79" s="2" t="s">
         <v>352</v>
@@ -5399,7 +5400,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="80" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
         <v>290</v>
       </c>
@@ -5437,7 +5438,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="81" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
         <v>291</v>
       </c>
@@ -5460,7 +5461,7 @@
         <v>4</v>
       </c>
       <c r="K81" s="3" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="L81" s="3" t="s">
         <v>352</v>
@@ -5472,7 +5473,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="82" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:21" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
         <v>292</v>
       </c>
@@ -5510,7 +5511,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="83" spans="1:21" ht="115.2" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:21" ht="115.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
         <v>293</v>
       </c>
@@ -5536,7 +5537,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="84" spans="1:21" ht="115.2" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:21" ht="115.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
         <v>294</v>
       </c>
@@ -5577,7 +5578,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="85" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
         <v>295</v>
       </c>
@@ -5609,7 +5610,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="86" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
         <v>296</v>
       </c>
@@ -5641,7 +5642,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="87" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
         <v>297</v>
       </c>
@@ -5673,7 +5674,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="88" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
         <v>298</v>
       </c>
@@ -5711,7 +5712,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="89" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" s="2" t="s">
         <v>299</v>
       </c>
@@ -5746,7 +5747,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="90" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
         <v>300</v>
       </c>
@@ -5781,7 +5782,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="91" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" s="2" t="s">
         <v>382</v>
       </c>
@@ -5819,7 +5820,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="92" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" s="2" t="s">
         <v>301</v>
       </c>
@@ -5845,7 +5846,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="93" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" s="2" t="s">
         <v>302</v>
       </c>
@@ -5933,7 +5934,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="95" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" s="2" t="s">
         <v>304</v>
       </c>
@@ -5974,7 +5975,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="96" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96" s="2" t="s">
         <v>305</v>
       </c>
@@ -6009,7 +6010,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="97" spans="1:21" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:21" ht="129.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" s="2" t="s">
         <v>306</v>
       </c>
@@ -6041,7 +6042,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="98" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" s="2" t="s">
         <v>307</v>
       </c>
@@ -6117,7 +6118,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="100" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" s="2" t="s">
         <v>309</v>
       </c>
@@ -6155,7 +6156,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="101" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" s="2" t="s">
         <v>310</v>
       </c>
@@ -6190,7 +6191,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="102" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" s="2" t="s">
         <v>311</v>
       </c>
@@ -6225,7 +6226,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="103" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" s="2" t="s">
         <v>312</v>
       </c>
@@ -6263,7 +6264,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="104" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" s="2" t="s">
         <v>313</v>
       </c>
@@ -6307,7 +6308,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="105" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" s="2" t="s">
         <v>314</v>
       </c>
@@ -6336,7 +6337,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="106" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" s="2" t="s">
         <v>315</v>
       </c>
@@ -6380,7 +6381,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="107" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" s="2" t="s">
         <v>316</v>
       </c>
@@ -6421,7 +6422,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="108" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" s="2" t="s">
         <v>317</v>
       </c>
@@ -6465,7 +6466,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="109" spans="1:21" ht="72" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:21" ht="72" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" s="2" t="s">
         <v>318</v>
       </c>
@@ -6500,7 +6501,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="110" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" s="2" t="s">
         <v>319</v>
       </c>
@@ -6523,7 +6524,7 @@
         <v>7</v>
       </c>
       <c r="K110" s="9" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="L110" s="10" t="s">
         <v>352</v>
@@ -6538,7 +6539,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="111" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" s="2" t="s">
         <v>320</v>
       </c>
@@ -6573,7 +6574,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="112" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:21" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A112" s="2" t="s">
         <v>321</v>
       </c>
@@ -6612,7 +6613,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="113" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" s="2" t="s">
         <v>322</v>
       </c>
@@ -6647,7 +6648,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="114" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" s="2" t="s">
         <v>323</v>
       </c>
@@ -6682,7 +6683,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="115" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:21" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" s="2" t="s">
         <v>324</v>
       </c>
@@ -6705,7 +6706,7 @@
         <v>1</v>
       </c>
       <c r="K115" s="3" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="L115" s="3" t="s">
         <v>352</v>
@@ -6720,7 +6721,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="116" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" s="2" t="s">
         <v>325</v>
       </c>
@@ -6761,7 +6762,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="117" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" s="2" t="s">
         <v>326</v>
       </c>
@@ -6789,7 +6790,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="118" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" s="2" t="s">
         <v>327</v>
       </c>
@@ -6814,7 +6815,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="119" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" s="2" t="s">
         <v>328</v>
       </c>
@@ -6852,7 +6853,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="120" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" s="2" t="s">
         <v>329</v>
       </c>
@@ -6893,7 +6894,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="121" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121" s="2" t="s">
         <v>330</v>
       </c>
@@ -6916,7 +6917,7 @@
         <v>4</v>
       </c>
       <c r="K121" s="2" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="L121" s="2" t="s">
         <v>352</v>
@@ -6928,7 +6929,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="122" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122" s="2" t="s">
         <v>331</v>
       </c>
@@ -6963,7 +6964,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="123" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" s="2" t="s">
         <v>332</v>
       </c>
@@ -6998,7 +6999,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="124" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" s="2" t="s">
         <v>333</v>
       </c>
@@ -7042,7 +7043,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="125" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" s="2" t="s">
         <v>334</v>
       </c>
@@ -7086,7 +7087,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="126" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126" s="2" t="s">
         <v>335</v>
       </c>
@@ -7127,7 +7128,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="127" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:21" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127" s="2" t="s">
         <v>336</v>
       </c>
@@ -7162,7 +7163,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="128" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128" s="2" t="s">
         <v>337</v>
       </c>
@@ -7197,7 +7198,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="129" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129" s="2" t="s">
         <v>338</v>
       </c>
@@ -7229,7 +7230,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="130" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" s="2" t="s">
         <v>339</v>
       </c>
@@ -7270,7 +7271,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="131" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" s="2" t="s">
         <v>340</v>
       </c>
@@ -7311,7 +7312,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="132" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132" s="2" t="s">
         <v>341</v>
       </c>
@@ -7358,7 +7359,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="133" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133" s="2" t="s">
         <v>342</v>
       </c>
@@ -7397,7 +7398,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="134" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134" s="2" t="s">
         <v>343</v>
       </c>
@@ -7436,7 +7437,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="135" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" s="2" t="s">
         <v>344</v>
       </c>
@@ -7480,7 +7481,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="136" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136" s="2" t="s">
         <v>345</v>
       </c>
@@ -7518,7 +7519,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="137" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137" s="2" t="s">
         <v>346</v>
       </c>
@@ -7553,7 +7554,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="138" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138" s="2" t="s">
         <v>347</v>
       </c>
@@ -7585,7 +7586,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="139" spans="1:21" ht="72" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:21" ht="72" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139" s="2" t="s">
         <v>348</v>
       </c>
@@ -7623,7 +7624,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="140" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:21" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140" s="2" t="s">
         <v>349</v>
       </c>
@@ -7649,7 +7650,7 @@
         <v>1</v>
       </c>
       <c r="K140" s="3" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="L140" s="2" t="s">
         <v>352</v>
@@ -7661,7 +7662,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="141" spans="1:21" ht="72" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:21" ht="72" hidden="1" x14ac:dyDescent="0.3">
       <c r="A141" s="2" t="s">
         <v>350</v>
       </c>
@@ -7684,7 +7685,7 @@
         <v>4</v>
       </c>
       <c r="K141" s="3" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="L141" s="3" t="s">
         <v>352</v>
@@ -7699,7 +7700,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="142" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A142" s="2" t="s">
         <v>359</v>
       </c>
@@ -7734,7 +7735,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="143" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143" s="2" t="s">
         <v>386</v>
       </c>
@@ -7769,7 +7770,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="144" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144" s="2" t="s">
         <v>387</v>
       </c>
@@ -7801,7 +7802,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="145" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A145" s="2" t="s">
         <v>388</v>
       </c>
@@ -7868,7 +7869,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="147" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A147" s="2" t="s">
         <v>451</v>
       </c>
@@ -7900,7 +7901,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="148" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A148" s="2" t="s">
         <v>400</v>
       </c>
@@ -7926,7 +7927,7 @@
         <v>407</v>
       </c>
       <c r="K148" s="2" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="L148" s="2" t="s">
         <v>352</v>
@@ -7938,7 +7939,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="149" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A149" s="2" t="s">
         <v>439</v>
       </c>
@@ -7970,7 +7971,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="150" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150" s="2" t="s">
         <v>453</v>
       </c>
@@ -8002,7 +8003,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="151" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151" s="2" t="s">
         <v>454</v>
       </c>
@@ -8034,7 +8035,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="152" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A152" s="2" t="s">
         <v>455</v>
       </c>
@@ -8066,7 +8067,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="153" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153" s="2" t="s">
         <v>456</v>
       </c>
@@ -8101,7 +8102,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="154" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154" s="2" t="s">
         <v>461</v>
       </c>
@@ -8130,7 +8131,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="155" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155" s="2" t="s">
         <v>483</v>
       </c>
@@ -8156,7 +8157,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="156" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156" s="2" t="s">
         <v>584</v>
       </c>
@@ -8194,14 +8195,20 @@
         <v>437</v>
       </c>
       <c r="R156" s="2" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="U156" s="2" t="s">
         <v>587</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V156" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:V156" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <filterColumn colId="9">
+      <filters>
+        <filter val="2"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N146">
     <sortCondition ref="E2:E146"/>
     <sortCondition ref="I2:I146"/>

</xml_diff>

<commit_message>
ov2 tried no success
</commit_message>
<xml_diff>
--- a/src/sastadev/data/methods/TARSP_Index_Current.xlsx
+++ b/src/sastadev/data/methods/TARSP_Index_Current.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\jodijk\myprograms\python\sastacode\mysastadev\src\sastadev\data\methods\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECD5D6FA-6ED0-47A6-B6D9-229F7178F3B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12F17369-7381-489B-B67E-98C1FC781562}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1611" uniqueCount="612">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1612" uniqueCount="613">
   <si>
     <t>Item</t>
   </si>
@@ -1139,11 +1139,6 @@
   </si>
   <si>
     <t>geenX</t>
-  </si>
-  <si>
-    <t>//node[@cat="np" and
-    node[@pt="vnw" and @rel="det" and @lemma="geen"] and
-    node[@pt="n" and @rel="hd"]]</t>
   </si>
   <si>
     <t>PV-loos</t>
@@ -1550,9 +1545,6 @@
 ]</t>
   </si>
   <si>
-    <t>//node[@cat="np" and node[@rel="det" and @lemma="de"] and count(node)=2]</t>
-  </si>
-  <si>
     <t>v.u.soc.divers,vu divers,vu soc divers, DIV</t>
   </si>
   <si>
@@ -1681,9 +1673,6 @@
     <t>//node[%FullOnd%]</t>
   </si>
   <si>
-    <t>//node[@pt="vg" and @lemma="en" and @rel="dlink"]</t>
-  </si>
-  <si>
     <t>//node[@lemma="hem" and @pt="vnw"]</t>
   </si>
   <si>
@@ -1825,12 +1814,6 @@
     <t>WOndX</t>
   </si>
   <si>
-    <t>//node[node[@rel="hd" and @pt="vz"] and 
-       node[@rel="obj1" and 
-            ( (@pt="vz" or @pt="bw") or 
-              (%Rpronoun% and @begin&gt;=../node[@rel="hd"]/@end)) ]]</t>
-  </si>
-  <si>
     <t>T166</t>
   </si>
   <si>
@@ -1867,9 +1850,6 @@
     <t>//node[%VzBepBvZn%]</t>
   </si>
   <si>
-    <t>//node[@pt="ww" and not(%verbal_VU%) and %thisistheonlyrealword%]</t>
-  </si>
-  <si>
     <t>//node[@lemma="jij" or (@lemma="je"  and (@vwtype="pr" or @vwtype="pers") and (@rel="su" )) and not(../node[%dankje_VU%])]</t>
   </si>
   <si>
@@ -1882,28 +1862,12 @@
     <t>//node[(@rel="mod" or @rel="dp")  and @cat="cp" and not(%Tarsp_ofmod%) and  not(%Tarsp_datmod%) and node[@rel="body" and node[@pt="ww" and @pvagr and @rel="hd"]]]</t>
   </si>
   <si>
-    <t>//node[@cat="np" and node[(@pt="n" or %substantivised_nphead%)  and @rel="hd"] and node[@pt="vnw" and @vwtype="aanw" and @rel="det" and (@lemma="dit" or @lemma="dat")] and count(node)=2]</t>
-  </si>
-  <si>
-    <t>//node[@cat="np" and node[(@pt="n" or %substantivised_nphead%) and @rel="hd"] and node[@pt="vnw" and @vwtype="aanw" and @rel="det" and (@lemma="die" or @lemma="deze")] and 
-count(node)=2]</t>
-  </si>
-  <si>
-    <t>//node[(node[@pt="n" and @rel="hd"] and node[@pt="n" and not(@rel="hd")] and count(node) = 2) or
-       (@cat="du" and count(node[@rel="dp" and @pt="n"]) = 2)]</t>
-  </si>
-  <si>
     <t>//node[@rel="svp" and @pt and not(%svpofhww%) and not(%advsvpofww%) and parent::node[node[@pt="ww" and contains(@lemma,"_") and @rel ="hd"]]]</t>
   </si>
   <si>
     <t>into</t>
   </si>
   <si>
-    <t>//node[@cat="np" and
-    node[@pt="lid" and @rel="det" and @lemma="het"] and
-    node[@rel="hd" and @pt="n"] and count(node)=2]</t>
-  </si>
-  <si>
     <t>stam</t>
   </si>
   <si>
@@ -1917,6 +1881,36 @@
   </si>
   <si>
     <t>//node[%Tarsp_een%]</t>
+  </si>
+  <si>
+    <t>//node[%Tarsp_die_deze_Zn%]</t>
+  </si>
+  <si>
+    <t>//node[%Tarsp_de%]</t>
+  </si>
+  <si>
+    <t>//node[%Tarsp_dit_dat_Zn%]</t>
+  </si>
+  <si>
+    <t>//node[%Tarsp_geen_X%]</t>
+  </si>
+  <si>
+    <t>//node[%Tarsp_het_Zn%]</t>
+  </si>
+  <si>
+    <t>//node[%Tarsp_Vz_B%]</t>
+  </si>
+  <si>
+    <t>//node[%Tarsp_ZnZn%]</t>
+  </si>
+  <si>
+    <t>//node[%Tarsp_only_W%]</t>
+  </si>
+  <si>
+    <t>//node[%Tarsp_en%]</t>
+  </si>
+  <si>
+    <t>intentionally not defined</t>
   </si>
 </sst>
 </file>
@@ -2038,9 +2032,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2078,7 +2072,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2184,7 +2178,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2326,7 +2320,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2334,7 +2328,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:V156"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2388,37 +2381,37 @@
         <v>157</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="P1" s="1" t="s">
+        <v>539</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>540</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>541</v>
+      </c>
+      <c r="S1" s="1" t="s">
         <v>542</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>543</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>545</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>546</v>
       </c>
       <c r="U1" s="1" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="2" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>212</v>
       </c>
@@ -2432,13 +2425,13 @@
         <v>192</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>70</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>352</v>
@@ -2450,7 +2443,7 @@
         <v>3</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>352</v>
@@ -2459,13 +2452,13 @@
         <v>353</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="3" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>213</v>
       </c>
@@ -2491,7 +2484,7 @@
         <v>6</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="L3" s="2" t="s">
         <v>352</v>
@@ -2500,13 +2493,13 @@
         <v>352</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U3" s="2" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="4" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>214</v>
       </c>
@@ -2520,7 +2513,7 @@
         <v>192</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>63</v>
@@ -2541,13 +2534,13 @@
         <v>353</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="R4" s="2" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="5" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>215</v>
       </c>
@@ -2579,13 +2572,13 @@
         <v>353</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U5" s="2" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="6" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>216</v>
       </c>
@@ -2608,7 +2601,7 @@
         <v>1</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>610</v>
+        <v>601</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>352</v>
@@ -2617,16 +2610,16 @@
         <v>353</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U6" s="2" t="s">
         <v>358</v>
       </c>
       <c r="V6" s="2" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="7" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>217</v>
       </c>
@@ -2637,7 +2630,7 @@
         <v>192</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>352</v>
@@ -2649,7 +2642,7 @@
         <v>1</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="L7" s="2" t="s">
         <v>353</v>
@@ -2658,10 +2651,10 @@
         <v>353</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="8" spans="1:22" ht="115.2" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>218</v>
       </c>
@@ -2687,7 +2680,7 @@
         <v>4</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="L8" s="3" t="s">
         <v>353</v>
@@ -2696,10 +2689,10 @@
         <v>353</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="9" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>219</v>
       </c>
@@ -2725,7 +2718,7 @@
         <v>6</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>600</v>
+        <v>595</v>
       </c>
       <c r="L9" s="2" t="s">
         <v>352</v>
@@ -2734,13 +2727,13 @@
         <v>352</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U9" s="2" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="10" spans="1:22" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>220</v>
       </c>
@@ -2763,7 +2756,7 @@
         <v>4</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="L10" s="3" t="s">
         <v>352</v>
@@ -2772,10 +2765,10 @@
         <v>353</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="11" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>221</v>
       </c>
@@ -2807,10 +2800,10 @@
         <v>353</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="12" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>222</v>
       </c>
@@ -2827,7 +2820,7 @@
         <v>38</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>352</v>
@@ -2839,7 +2832,7 @@
         <v>3</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>588</v>
+        <v>584</v>
       </c>
       <c r="L12" s="2" t="s">
         <v>352</v>
@@ -2848,10 +2841,10 @@
         <v>353</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="13" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>223</v>
       </c>
@@ -2874,7 +2867,7 @@
         <v>5</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>590</v>
+        <v>586</v>
       </c>
       <c r="L13" s="3" t="s">
         <v>352</v>
@@ -2883,10 +2876,10 @@
         <v>353</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>224</v>
       </c>
@@ -2912,7 +2905,7 @@
         <v>4</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L14" s="2" t="s">
         <v>353</v>
@@ -2921,10 +2914,10 @@
         <v>353</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>225</v>
       </c>
@@ -2947,7 +2940,7 @@
         <v>4</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="L15" s="2" t="s">
         <v>352</v>
@@ -2956,10 +2949,10 @@
         <v>353</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>226</v>
       </c>
@@ -2976,7 +2969,7 @@
         <v>352</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="L16" s="2" t="s">
         <v>353</v>
@@ -2985,10 +2978,10 @@
         <v>353</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="17" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>227</v>
       </c>
@@ -3017,10 +3010,10 @@
         <v>352</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="18" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>228</v>
       </c>
@@ -3034,10 +3027,10 @@
         <v>192</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="H18" s="2" t="s">
         <v>352</v>
@@ -3055,13 +3048,13 @@
         <v>353</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="P18" s="2" t="s">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="19" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="19" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>229</v>
       </c>
@@ -3072,10 +3065,10 @@
         <v>192</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>352</v>
@@ -3087,7 +3080,7 @@
         <v>1</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>589</v>
+        <v>585</v>
       </c>
       <c r="L19" s="2" t="s">
         <v>352</v>
@@ -3096,10 +3089,10 @@
         <v>352</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="20" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>230</v>
       </c>
@@ -3128,10 +3121,10 @@
         <v>353</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="21" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="21" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>231</v>
       </c>
@@ -3154,7 +3147,7 @@
         <v>4</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>591</v>
+        <v>587</v>
       </c>
       <c r="L21" s="2" t="s">
         <v>352</v>
@@ -3163,10 +3156,10 @@
         <v>353</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="22" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="22" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>232</v>
       </c>
@@ -3189,7 +3182,7 @@
         <v>3</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="L22" s="2" t="s">
         <v>352</v>
@@ -3198,10 +3191,10 @@
         <v>353</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="23" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="23" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>233</v>
       </c>
@@ -3218,7 +3211,7 @@
         <v>47</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="H23" s="2" t="s">
         <v>352</v>
@@ -3230,7 +3223,7 @@
         <v>5</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="L23" s="2" t="s">
         <v>352</v>
@@ -3239,7 +3232,7 @@
         <v>353</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="24" spans="1:21" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -3256,13 +3249,13 @@
         <v>192</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>26</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
       <c r="H24" s="2" t="s">
         <v>352</v>
@@ -3274,7 +3267,7 @@
         <v>2</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>608</v>
+        <v>599</v>
       </c>
       <c r="L24" s="2" t="s">
         <v>352</v>
@@ -3283,13 +3276,13 @@
         <v>353</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U24" s="3" t="s">
-        <v>493</v>
-      </c>
-    </row>
-    <row r="25" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="25" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>235</v>
       </c>
@@ -3318,10 +3311,10 @@
         <v>353</v>
       </c>
       <c r="N25" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="26" spans="1:21" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="26" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>236</v>
       </c>
@@ -3344,7 +3337,7 @@
         <v>4</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>494</v>
+        <v>604</v>
       </c>
       <c r="L26" s="3" t="s">
         <v>352</v>
@@ -3353,13 +3346,13 @@
         <v>353</v>
       </c>
       <c r="N26" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U26" s="2" t="s">
-        <v>471</v>
-      </c>
-    </row>
-    <row r="27" spans="1:21" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="27" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>237</v>
       </c>
@@ -3382,7 +3375,7 @@
         <v>4</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="L27" s="2" t="s">
         <v>352</v>
@@ -3391,10 +3384,10 @@
         <v>353</v>
       </c>
       <c r="N27" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="28" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="28" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>238</v>
       </c>
@@ -3417,7 +3410,7 @@
         <v>5</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
       <c r="L28" s="2" t="s">
         <v>352</v>
@@ -3426,7 +3419,7 @@
         <v>352</v>
       </c>
       <c r="N28" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.3">
@@ -3452,7 +3445,7 @@
         <v>2</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>611</v>
+        <v>602</v>
       </c>
       <c r="L29" s="2" t="s">
         <v>352</v>
@@ -3461,13 +3454,13 @@
         <v>353</v>
       </c>
       <c r="N29" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U29" s="2" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="30" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="30" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>240</v>
       </c>
@@ -3490,7 +3483,7 @@
         <v>3</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>536</v>
+        <v>611</v>
       </c>
       <c r="L30" s="2" t="s">
         <v>352</v>
@@ -3499,13 +3492,13 @@
         <v>352</v>
       </c>
       <c r="N30" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U30" s="2" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="31" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>241</v>
       </c>
@@ -3537,13 +3530,13 @@
         <v>353</v>
       </c>
       <c r="N31" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="R31" s="2" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="32" spans="1:21" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="32" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>242</v>
       </c>
@@ -3569,7 +3562,7 @@
         <v>6</v>
       </c>
       <c r="K32" s="3" t="s">
-        <v>365</v>
+        <v>606</v>
       </c>
       <c r="L32" s="3" t="s">
         <v>352</v>
@@ -3578,10 +3571,10 @@
         <v>353</v>
       </c>
       <c r="N32" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="33" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="33" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>243</v>
       </c>
@@ -3610,7 +3603,7 @@
         <v>3</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>576</v>
+        <v>573</v>
       </c>
       <c r="L33" s="2" t="s">
         <v>352</v>
@@ -3619,13 +3612,13 @@
         <v>353</v>
       </c>
       <c r="N33" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="R33" s="2" t="s">
-        <v>581</v>
-      </c>
-    </row>
-    <row r="34" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="34" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>244</v>
       </c>
@@ -3648,7 +3641,7 @@
         <v>6</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="L34" s="2" t="s">
         <v>352</v>
@@ -3657,10 +3650,10 @@
         <v>353</v>
       </c>
       <c r="N34" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="35" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="35" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>245</v>
       </c>
@@ -3692,10 +3685,10 @@
         <v>352</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="36" spans="1:21" ht="72" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="36" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>246</v>
       </c>
@@ -3718,7 +3711,7 @@
         <v>5</v>
       </c>
       <c r="K36" s="3" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="L36" s="3" t="s">
         <v>352</v>
@@ -3727,10 +3720,10 @@
         <v>352</v>
       </c>
       <c r="N36" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="37" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="37" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>247</v>
       </c>
@@ -3753,7 +3746,7 @@
         <v>3</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="L37" s="2" t="s">
         <v>352</v>
@@ -3762,10 +3755,10 @@
         <v>353</v>
       </c>
       <c r="N37" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="38" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="38" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>248</v>
       </c>
@@ -3782,7 +3775,7 @@
         <v>208</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="H38" s="2" t="s">
         <v>352</v>
@@ -3794,7 +3787,7 @@
         <v>362</v>
       </c>
       <c r="K38" s="3" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="L38" s="3" t="s">
         <v>352</v>
@@ -3803,10 +3796,10 @@
         <v>353</v>
       </c>
       <c r="N38" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="39" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="39" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>249</v>
       </c>
@@ -3823,7 +3816,7 @@
         <v>209</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="H39" s="2" t="s">
         <v>352</v>
@@ -3835,7 +3828,7 @@
         <v>4</v>
       </c>
       <c r="K39" s="3" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="L39" s="3" t="s">
         <v>352</v>
@@ -3844,10 +3837,10 @@
         <v>353</v>
       </c>
       <c r="N39" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="40" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="40" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>250</v>
       </c>
@@ -3861,7 +3854,7 @@
         <v>145</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="H40" s="2" t="s">
         <v>352</v>
@@ -3873,7 +3866,7 @@
         <v>3</v>
       </c>
       <c r="K40" s="3" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="L40" s="3" t="s">
         <v>352</v>
@@ -3882,13 +3875,13 @@
         <v>352</v>
       </c>
       <c r="N40" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U40" s="2" t="s">
-        <v>472</v>
-      </c>
-    </row>
-    <row r="41" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="41" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>251</v>
       </c>
@@ -3920,7 +3913,7 @@
         <v>352</v>
       </c>
       <c r="N41" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.3">
@@ -3940,7 +3933,7 @@
         <v>67</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="H42" s="2" t="s">
         <v>352</v>
@@ -3952,7 +3945,7 @@
         <v>2</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>605</v>
+        <v>597</v>
       </c>
       <c r="L42" s="2" t="s">
         <v>352</v>
@@ -3961,13 +3954,13 @@
         <v>353</v>
       </c>
       <c r="N42" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U42" s="2" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="43" spans="1:21" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>253</v>
       </c>
@@ -3981,10 +3974,10 @@
         <v>192</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="H43" s="2" t="s">
         <v>352</v>
@@ -3996,7 +3989,7 @@
         <v>3</v>
       </c>
       <c r="K43" s="3" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="L43" s="2" t="s">
         <v>352</v>
@@ -4005,13 +3998,13 @@
         <v>353</v>
       </c>
       <c r="N43" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U43" s="2" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="44" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>254</v>
       </c>
@@ -4034,7 +4027,7 @@
         <v>3</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>597</v>
+        <v>592</v>
       </c>
       <c r="L44" s="2" t="s">
         <v>352</v>
@@ -4043,10 +4036,10 @@
         <v>353</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="45" spans="1:21" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="45" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>255</v>
       </c>
@@ -4069,7 +4062,7 @@
         <v>6</v>
       </c>
       <c r="K45" s="3" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="L45" s="2" t="s">
         <v>352</v>
@@ -4078,7 +4071,7 @@
         <v>353</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.3">
@@ -4101,7 +4094,7 @@
         <v>201</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="H46" s="2" t="s">
         <v>352</v>
@@ -4113,7 +4106,7 @@
         <v>2</v>
       </c>
       <c r="K46" s="2" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="L46" s="2" t="s">
         <v>352</v>
@@ -4122,10 +4115,10 @@
         <v>353</v>
       </c>
       <c r="N46" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="47" spans="1:21" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="47" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>257</v>
       </c>
@@ -4148,7 +4141,7 @@
         <v>6</v>
       </c>
       <c r="K47" s="3" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="L47" s="2" t="s">
         <v>352</v>
@@ -4157,13 +4150,13 @@
         <v>353</v>
       </c>
       <c r="N47" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U47" s="2" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="48" spans="1:21" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>258</v>
       </c>
@@ -4177,7 +4170,7 @@
         <v>353</v>
       </c>
       <c r="K48" s="3" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="L48" s="3" t="s">
         <v>353</v>
@@ -4186,13 +4179,13 @@
         <v>353</v>
       </c>
       <c r="N48" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U48" s="6" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="49" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>259</v>
       </c>
@@ -4224,10 +4217,10 @@
         <v>353</v>
       </c>
       <c r="N49" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="50" spans="1:21" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="50" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>260</v>
       </c>
@@ -4250,7 +4243,7 @@
         <v>5</v>
       </c>
       <c r="K50" s="3" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="L50" s="2" t="s">
         <v>352</v>
@@ -4259,10 +4252,10 @@
         <v>353</v>
       </c>
       <c r="N50" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="51" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="51" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>261</v>
       </c>
@@ -4285,7 +4278,7 @@
         <v>4</v>
       </c>
       <c r="K51" s="2" t="s">
-        <v>573</v>
+        <v>570</v>
       </c>
       <c r="L51" s="2" t="s">
         <v>352</v>
@@ -4294,7 +4287,7 @@
         <v>353</v>
       </c>
       <c r="N51" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.3">
@@ -4323,7 +4316,7 @@
         <v>2</v>
       </c>
       <c r="K52" s="2" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="L52" s="2" t="s">
         <v>352</v>
@@ -4332,10 +4325,10 @@
         <v>353</v>
       </c>
       <c r="N52" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="53" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="53" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>263</v>
       </c>
@@ -4358,7 +4351,7 @@
         <v>6</v>
       </c>
       <c r="K53" s="2" t="s">
-        <v>594</v>
+        <v>590</v>
       </c>
       <c r="L53" s="2" t="s">
         <v>352</v>
@@ -4367,10 +4360,10 @@
         <v>353</v>
       </c>
       <c r="N53" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="54" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="54" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>264</v>
       </c>
@@ -4396,7 +4389,7 @@
         <v>6</v>
       </c>
       <c r="K54" s="2" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="L54" s="2" t="s">
         <v>352</v>
@@ -4405,10 +4398,10 @@
         <v>353</v>
       </c>
       <c r="N54" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="55" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="55" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>265</v>
       </c>
@@ -4440,10 +4433,10 @@
         <v>352</v>
       </c>
       <c r="N55" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="56" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="56" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>266</v>
       </c>
@@ -4472,13 +4465,13 @@
         <v>353</v>
       </c>
       <c r="N56" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="R56" s="2" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="57" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="57" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>267</v>
       </c>
@@ -4501,7 +4494,7 @@
         <v>1</v>
       </c>
       <c r="K57" s="3" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="L57" s="2" t="s">
         <v>353</v>
@@ -4510,7 +4503,7 @@
         <v>353</v>
       </c>
       <c r="N57" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.3">
@@ -4530,7 +4523,7 @@
         <v>21</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="H58" s="2" t="s">
         <v>352</v>
@@ -4542,7 +4535,7 @@
         <v>2</v>
       </c>
       <c r="K58" s="2" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="L58" s="2" t="s">
         <v>352</v>
@@ -4551,10 +4544,10 @@
         <v>352</v>
       </c>
       <c r="N58" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="59" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="59" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>269</v>
       </c>
@@ -4571,7 +4564,7 @@
         <v>39</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>552</v>
+        <v>549</v>
       </c>
       <c r="H59" s="2" t="s">
         <v>352</v>
@@ -4583,7 +4576,7 @@
         <v>3</v>
       </c>
       <c r="K59" s="2" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="L59" s="2" t="s">
         <v>352</v>
@@ -4592,10 +4585,10 @@
         <v>353</v>
       </c>
       <c r="N59" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="60" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="60" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>270</v>
       </c>
@@ -4609,7 +4602,7 @@
         <v>192</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F60" s="2" t="s">
         <v>65</v>
@@ -4630,13 +4623,13 @@
         <v>353</v>
       </c>
       <c r="N60" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="R60" s="2" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="61" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="61" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>271</v>
       </c>
@@ -4668,13 +4661,13 @@
         <v>353</v>
       </c>
       <c r="N61" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U61" s="2" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="62" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="62" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>272</v>
       </c>
@@ -4706,13 +4699,13 @@
         <v>353</v>
       </c>
       <c r="N62" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U62" s="2" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="63" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="63" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>273</v>
       </c>
@@ -4744,13 +4737,13 @@
         <v>353</v>
       </c>
       <c r="N63" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U63" s="2" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="64" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="64" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>274</v>
       </c>
@@ -4773,7 +4766,7 @@
         <v>4</v>
       </c>
       <c r="K64" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="L64" s="2" t="s">
         <v>353</v>
@@ -4782,7 +4775,7 @@
         <v>352</v>
       </c>
       <c r="N64" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.3">
@@ -4814,7 +4807,7 @@
         <v>2</v>
       </c>
       <c r="K65" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="L65" s="2" t="s">
         <v>352</v>
@@ -4823,7 +4816,7 @@
         <v>352</v>
       </c>
       <c r="N65" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.3">
@@ -4843,7 +4836,7 @@
         <v>25</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
       <c r="H66" s="2" t="s">
         <v>352</v>
@@ -4855,7 +4848,7 @@
         <v>2</v>
       </c>
       <c r="K66" s="2" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="L66" s="2" t="s">
         <v>352</v>
@@ -4864,10 +4857,10 @@
         <v>352</v>
       </c>
       <c r="N66" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="67" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="67" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>277</v>
       </c>
@@ -4884,7 +4877,7 @@
         <v>35</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="H67" s="2" t="s">
         <v>352</v>
@@ -4896,7 +4889,7 @@
         <v>3</v>
       </c>
       <c r="K67" s="3" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="L67" s="2" t="s">
         <v>352</v>
@@ -4905,10 +4898,10 @@
         <v>353</v>
       </c>
       <c r="N67" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="68" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="68" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>278</v>
       </c>
@@ -4925,7 +4918,7 @@
         <v>44</v>
       </c>
       <c r="G68" s="2" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
       <c r="H68" s="2" t="s">
         <v>352</v>
@@ -4937,7 +4930,7 @@
         <v>4</v>
       </c>
       <c r="K68" s="3" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="L68" s="2" t="s">
         <v>352</v>
@@ -4946,10 +4939,10 @@
         <v>353</v>
       </c>
       <c r="N68" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="69" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="69" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>279</v>
       </c>
@@ -4966,7 +4959,7 @@
         <v>43</v>
       </c>
       <c r="G69" s="2" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
       <c r="H69" s="2" t="s">
         <v>352</v>
@@ -4978,7 +4971,7 @@
         <v>4</v>
       </c>
       <c r="K69" s="3" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="L69" s="2" t="s">
         <v>352</v>
@@ -4987,10 +4980,10 @@
         <v>352</v>
       </c>
       <c r="N69" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="70" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="70" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>280</v>
       </c>
@@ -5007,7 +5000,7 @@
         <v>32</v>
       </c>
       <c r="G70" s="2" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="H70" s="2" t="s">
         <v>352</v>
@@ -5019,7 +5012,7 @@
         <v>3</v>
       </c>
       <c r="K70" s="3" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="L70" s="2" t="s">
         <v>352</v>
@@ -5028,10 +5021,10 @@
         <v>352</v>
       </c>
       <c r="N70" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="71" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="71" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>281</v>
       </c>
@@ -5048,7 +5041,7 @@
         <v>46</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
       <c r="H71" s="2" t="s">
         <v>352</v>
@@ -5060,7 +5053,7 @@
         <v>5</v>
       </c>
       <c r="K71" s="2" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="L71" s="2" t="s">
         <v>352</v>
@@ -5069,7 +5062,7 @@
         <v>352</v>
       </c>
       <c r="N71" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.3">
@@ -5086,13 +5079,13 @@
         <v>192</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="G72" s="2" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="H72" s="2" t="s">
         <v>352</v>
@@ -5110,10 +5103,13 @@
         <v>353</v>
       </c>
       <c r="N72" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="73" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+      <c r="U72" s="2" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="73" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>283</v>
       </c>
@@ -5130,10 +5126,10 @@
         <v>187</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="H73" s="2" t="s">
         <v>352</v>
@@ -5145,7 +5141,7 @@
         <v>3</v>
       </c>
       <c r="K73" s="2" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="L73" s="2" t="s">
         <v>352</v>
@@ -5154,10 +5150,10 @@
         <v>353</v>
       </c>
       <c r="N73" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="74" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="74" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
         <v>284</v>
       </c>
@@ -5174,7 +5170,7 @@
         <v>188</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="H74" s="2" t="s">
         <v>352</v>
@@ -5192,13 +5188,13 @@
         <v>353</v>
       </c>
       <c r="N74" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="R74" s="2" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="75" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="75" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
         <v>285</v>
       </c>
@@ -5227,13 +5223,13 @@
         <v>353</v>
       </c>
       <c r="N75" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="R75" s="2" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="76" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="76" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
         <v>286</v>
       </c>
@@ -5247,7 +5243,7 @@
         <v>190</v>
       </c>
       <c r="F76" s="2" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="H76" s="2" t="s">
         <v>352</v>
@@ -5265,13 +5261,13 @@
         <v>353</v>
       </c>
       <c r="N76" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U76" s="2" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="77" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
         <v>287</v>
       </c>
@@ -5288,10 +5284,10 @@
         <v>49</v>
       </c>
       <c r="F77" s="2" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="G77" s="2" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="H77" s="2" t="s">
         <v>352</v>
@@ -5303,7 +5299,7 @@
         <v>4</v>
       </c>
       <c r="K77" s="3" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="L77" s="2" t="s">
         <v>352</v>
@@ -5312,10 +5308,10 @@
         <v>353</v>
       </c>
       <c r="N77" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="78" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="78" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
         <v>288</v>
       </c>
@@ -5332,10 +5328,10 @@
         <v>48</v>
       </c>
       <c r="F78" s="2" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="G78" s="2" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="H78" s="2" t="s">
         <v>352</v>
@@ -5347,7 +5343,7 @@
         <v>5</v>
       </c>
       <c r="K78" s="3" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="L78" s="2" t="s">
         <v>352</v>
@@ -5356,10 +5352,10 @@
         <v>353</v>
       </c>
       <c r="N78" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="79" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="79" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
         <v>289</v>
       </c>
@@ -5373,7 +5369,7 @@
         <v>139</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="H79" s="2" t="s">
         <v>352</v>
@@ -5385,7 +5381,7 @@
         <v>6</v>
       </c>
       <c r="K79" s="2" t="s">
-        <v>598</v>
+        <v>593</v>
       </c>
       <c r="L79" s="2" t="s">
         <v>352</v>
@@ -5394,13 +5390,13 @@
         <v>353</v>
       </c>
       <c r="N79" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="R79" s="2" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="80" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="80" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
         <v>290</v>
       </c>
@@ -5432,13 +5428,13 @@
         <v>353</v>
       </c>
       <c r="N80" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U80" s="2" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="81" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
         <v>291</v>
       </c>
@@ -5461,7 +5457,7 @@
         <v>4</v>
       </c>
       <c r="K81" s="3" t="s">
-        <v>607</v>
+        <v>598</v>
       </c>
       <c r="L81" s="3" t="s">
         <v>352</v>
@@ -5470,10 +5466,10 @@
         <v>353</v>
       </c>
       <c r="N81" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="82" spans="1:21" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="82" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
         <v>292</v>
       </c>
@@ -5487,7 +5483,7 @@
         <v>150</v>
       </c>
       <c r="F82" s="2" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="H82" s="2" t="s">
         <v>352</v>
@@ -5499,7 +5495,7 @@
         <v>4</v>
       </c>
       <c r="K82" s="3" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="L82" s="2" t="s">
         <v>352</v>
@@ -5508,10 +5504,10 @@
         <v>353</v>
       </c>
       <c r="N82" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="83" spans="1:21" ht="115.2" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="83" spans="1:21" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
         <v>293</v>
       </c>
@@ -5534,10 +5530,10 @@
         <v>353</v>
       </c>
       <c r="N83" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="84" spans="1:21" ht="115.2" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="84" spans="1:21" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
         <v>294</v>
       </c>
@@ -5572,13 +5568,13 @@
         <v>353</v>
       </c>
       <c r="N84" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="R84" s="2" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="85" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="85" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
         <v>295</v>
       </c>
@@ -5607,10 +5603,10 @@
         <v>353</v>
       </c>
       <c r="N85" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="86" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="86" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
         <v>296</v>
       </c>
@@ -5639,10 +5635,10 @@
         <v>353</v>
       </c>
       <c r="N86" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="87" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="87" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
         <v>297</v>
       </c>
@@ -5671,10 +5667,10 @@
         <v>353</v>
       </c>
       <c r="N87" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="88" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="88" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
         <v>298</v>
       </c>
@@ -5685,10 +5681,10 @@
         <v>192</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="H88" s="2" t="s">
         <v>352</v>
@@ -5700,7 +5696,7 @@
         <v>1</v>
       </c>
       <c r="K88" s="3" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
       <c r="L88" s="2" t="s">
         <v>352</v>
@@ -5709,10 +5705,10 @@
         <v>353</v>
       </c>
       <c r="N88" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="89" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="89" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A89" s="2" t="s">
         <v>299</v>
       </c>
@@ -5723,7 +5719,7 @@
         <v>192</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="H89" s="2" t="s">
         <v>352</v>
@@ -5735,7 +5731,7 @@
         <v>1</v>
       </c>
       <c r="K89" s="2" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="L89" s="2" t="s">
         <v>352</v>
@@ -5744,10 +5740,10 @@
         <v>353</v>
       </c>
       <c r="N89" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="90" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="90" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
         <v>300</v>
       </c>
@@ -5758,10 +5754,10 @@
         <v>192</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="F90" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="H90" s="2" t="s">
         <v>352</v>
@@ -5779,12 +5775,12 @@
         <v>353</v>
       </c>
       <c r="N90" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="91" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="91" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A91" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B91" s="2" t="s">
         <v>2</v>
@@ -5793,22 +5789,22 @@
         <v>192</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="F91" s="2" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="H91" s="2" t="s">
         <v>352</v>
       </c>
       <c r="I91" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="J91" s="2" t="s">
         <v>380</v>
       </c>
-      <c r="J91" s="2" t="s">
-        <v>381</v>
-      </c>
       <c r="K91" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="L91" s="2" t="s">
         <v>352</v>
@@ -5817,10 +5813,10 @@
         <v>353</v>
       </c>
       <c r="N91" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="92" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="92" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A92" s="2" t="s">
         <v>301</v>
       </c>
@@ -5834,7 +5830,7 @@
         <v>352</v>
       </c>
       <c r="K92" s="2" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="L92" s="2" t="s">
         <v>353</v>
@@ -5843,10 +5839,10 @@
         <v>353</v>
       </c>
       <c r="N92" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="93" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="93" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A93" s="2" t="s">
         <v>302</v>
       </c>
@@ -5863,7 +5859,7 @@
         <v>59</v>
       </c>
       <c r="F93" s="2" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="H93" s="2" t="s">
         <v>352</v>
@@ -5875,7 +5871,7 @@
         <v>6</v>
       </c>
       <c r="K93" s="2" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="L93" s="2" t="s">
         <v>352</v>
@@ -5884,7 +5880,7 @@
         <v>352</v>
       </c>
       <c r="N93" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="94" spans="1:21" x14ac:dyDescent="0.3">
@@ -5904,10 +5900,10 @@
         <v>24</v>
       </c>
       <c r="F94" s="2" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
       <c r="G94" s="2" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="H94" s="2" t="s">
         <v>352</v>
@@ -5919,7 +5915,7 @@
         <v>2</v>
       </c>
       <c r="K94" s="2" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="L94" s="2" t="s">
         <v>352</v>
@@ -5928,13 +5924,13 @@
         <v>352</v>
       </c>
       <c r="N94" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U94" s="2" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="95" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A95" s="2" t="s">
         <v>304</v>
       </c>
@@ -5951,7 +5947,7 @@
         <v>45</v>
       </c>
       <c r="G95" s="2" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
       <c r="H95" s="2" t="s">
         <v>352</v>
@@ -5963,7 +5959,7 @@
         <v>5</v>
       </c>
       <c r="K95" s="2" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="L95" s="2" t="s">
         <v>352</v>
@@ -5972,10 +5968,10 @@
         <v>352</v>
       </c>
       <c r="N95" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="96" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="96" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A96" s="2" t="s">
         <v>305</v>
       </c>
@@ -5998,7 +5994,7 @@
         <v>3</v>
       </c>
       <c r="K96" s="2" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="L96" s="2" t="s">
         <v>353</v>
@@ -6007,10 +6003,10 @@
         <v>352</v>
       </c>
       <c r="N96" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="97" spans="1:21" ht="129.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="97" spans="1:21" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A97" s="2" t="s">
         <v>306</v>
       </c>
@@ -6024,13 +6020,13 @@
         <v>352</v>
       </c>
       <c r="I97" s="2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="J97" s="2" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="K97" s="3" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="L97" s="3" t="s">
         <v>352</v>
@@ -6039,10 +6035,10 @@
         <v>353</v>
       </c>
       <c r="N97" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="98" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="98" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A98" s="2" t="s">
         <v>307</v>
       </c>
@@ -6071,10 +6067,10 @@
         <v>353</v>
       </c>
       <c r="N98" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="R98" s="2" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
     </row>
     <row r="99" spans="1:21" x14ac:dyDescent="0.3">
@@ -6088,7 +6084,7 @@
         <v>194</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="F99" s="2" t="s">
         <v>142</v>
@@ -6103,7 +6099,7 @@
         <v>2</v>
       </c>
       <c r="K99" s="2" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
       <c r="L99" s="2" t="s">
         <v>352</v>
@@ -6112,13 +6108,13 @@
         <v>353</v>
       </c>
       <c r="N99" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="P99" s="2" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="100" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="100" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A100" s="2" t="s">
         <v>309</v>
       </c>
@@ -6132,7 +6128,7 @@
         <v>153</v>
       </c>
       <c r="F100" s="2" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="H100" s="2" t="s">
         <v>352</v>
@@ -6144,7 +6140,7 @@
         <v>6</v>
       </c>
       <c r="K100" s="2" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="L100" s="2" t="s">
         <v>352</v>
@@ -6153,10 +6149,10 @@
         <v>352</v>
       </c>
       <c r="N100" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="101" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="101" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A101" s="2" t="s">
         <v>310</v>
       </c>
@@ -6179,7 +6175,7 @@
         <v>5</v>
       </c>
       <c r="K101" s="3" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="L101" s="2" t="s">
         <v>352</v>
@@ -6188,10 +6184,10 @@
         <v>353</v>
       </c>
       <c r="N101" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="102" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="102" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A102" s="2" t="s">
         <v>311</v>
       </c>
@@ -6214,7 +6210,7 @@
         <v>4</v>
       </c>
       <c r="K102" s="2" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="L102" s="2" t="s">
         <v>352</v>
@@ -6223,10 +6219,10 @@
         <v>353</v>
       </c>
       <c r="N102" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="103" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="103" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A103" s="2" t="s">
         <v>312</v>
       </c>
@@ -6261,10 +6257,10 @@
         <v>353</v>
       </c>
       <c r="N103" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="104" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="104" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A104" s="2" t="s">
         <v>313</v>
       </c>
@@ -6275,10 +6271,10 @@
         <v>194</v>
       </c>
       <c r="E104" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F104" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="H104" s="2" t="s">
         <v>352</v>
@@ -6296,19 +6292,19 @@
         <v>353</v>
       </c>
       <c r="N104" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="P104" s="2" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="R104" s="2" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="U104" s="2" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="105" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A105" s="2" t="s">
         <v>314</v>
       </c>
@@ -6331,13 +6327,13 @@
         <v>353</v>
       </c>
       <c r="N105" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U105" s="2" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="106" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A106" s="2" t="s">
         <v>315</v>
       </c>
@@ -6366,7 +6362,7 @@
         <v>4</v>
       </c>
       <c r="K106" s="3" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="L106" s="2" t="s">
         <v>352</v>
@@ -6375,13 +6371,13 @@
         <v>353</v>
       </c>
       <c r="N106" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U106" s="2" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="107" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A107" s="2" t="s">
         <v>316</v>
       </c>
@@ -6407,7 +6403,7 @@
         <v>5</v>
       </c>
       <c r="K107" s="3" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="L107" s="2" t="s">
         <v>352</v>
@@ -6416,13 +6412,13 @@
         <v>353</v>
       </c>
       <c r="N107" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U107" s="2" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="108" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="108" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A108" s="2" t="s">
         <v>317</v>
       </c>
@@ -6448,7 +6444,7 @@
         <v>6</v>
       </c>
       <c r="K108" s="2" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="L108" s="2" t="s">
         <v>352</v>
@@ -6457,16 +6453,16 @@
         <v>352</v>
       </c>
       <c r="N108" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="P108" s="2" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="U108" s="2" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="109" spans="1:21" ht="72" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A109" s="2" t="s">
         <v>318</v>
       </c>
@@ -6489,7 +6485,7 @@
         <v>6</v>
       </c>
       <c r="K109" s="3" t="s">
-        <v>583</v>
+        <v>608</v>
       </c>
       <c r="L109" s="2" t="s">
         <v>352</v>
@@ -6498,10 +6494,10 @@
         <v>353</v>
       </c>
       <c r="N109" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="110" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="110" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A110" s="2" t="s">
         <v>319</v>
       </c>
@@ -6524,7 +6520,7 @@
         <v>7</v>
       </c>
       <c r="K110" s="9" t="s">
-        <v>595</v>
+        <v>591</v>
       </c>
       <c r="L110" s="10" t="s">
         <v>352</v>
@@ -6533,13 +6529,13 @@
         <v>353</v>
       </c>
       <c r="N110" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="R110" s="2" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="111" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="111" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A111" s="2" t="s">
         <v>320</v>
       </c>
@@ -6562,7 +6558,7 @@
         <v>4</v>
       </c>
       <c r="K111" s="2" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="L111" s="2" t="s">
         <v>352</v>
@@ -6571,10 +6567,10 @@
         <v>352</v>
       </c>
       <c r="N111" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="112" spans="1:21" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="112" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A112" s="2" t="s">
         <v>321</v>
       </c>
@@ -6598,7 +6594,7 @@
         <v>3</v>
       </c>
       <c r="K112" s="2" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="L112" s="2" t="s">
         <v>352</v>
@@ -6607,13 +6603,13 @@
         <v>353</v>
       </c>
       <c r="N112" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U112" s="3" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="113" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="113" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A113" s="2" t="s">
         <v>322</v>
       </c>
@@ -6645,10 +6641,10 @@
         <v>353</v>
       </c>
       <c r="N113" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="114" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="114" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A114" s="2" t="s">
         <v>323</v>
       </c>
@@ -6659,7 +6655,7 @@
         <v>192</v>
       </c>
       <c r="E114" s="2" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="H114" s="2" t="s">
         <v>352</v>
@@ -6671,7 +6667,7 @@
         <v>1</v>
       </c>
       <c r="K114" s="3" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="L114" s="2" t="s">
         <v>353</v>
@@ -6680,10 +6676,10 @@
         <v>352</v>
       </c>
       <c r="N114" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="115" spans="1:21" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="115" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A115" s="2" t="s">
         <v>324</v>
       </c>
@@ -6706,7 +6702,7 @@
         <v>1</v>
       </c>
       <c r="K115" s="3" t="s">
-        <v>596</v>
+        <v>610</v>
       </c>
       <c r="L115" s="3" t="s">
         <v>352</v>
@@ -6715,13 +6711,13 @@
         <v>353</v>
       </c>
       <c r="N115" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U115" s="2" t="s">
-        <v>477</v>
-      </c>
-    </row>
-    <row r="116" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="116" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A116" s="2" t="s">
         <v>325</v>
       </c>
@@ -6738,7 +6734,7 @@
         <v>79</v>
       </c>
       <c r="G116" s="2" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="H116" s="2" t="s">
         <v>352</v>
@@ -6750,7 +6746,7 @@
         <v>3</v>
       </c>
       <c r="K116" s="2" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="L116" s="2" t="s">
         <v>352</v>
@@ -6759,10 +6755,10 @@
         <v>353</v>
       </c>
       <c r="N116" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="117" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="117" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A117" s="2" t="s">
         <v>326</v>
       </c>
@@ -6770,7 +6766,7 @@
         <v>192</v>
       </c>
       <c r="E117" s="4" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="F117" s="4"/>
       <c r="G117" s="4"/>
@@ -6787,10 +6783,10 @@
         <v>353</v>
       </c>
       <c r="N117" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="118" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="118" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A118" s="2" t="s">
         <v>327</v>
       </c>
@@ -6812,10 +6808,10 @@
         <v>353</v>
       </c>
       <c r="N118" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="119" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="119" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A119" s="2" t="s">
         <v>328</v>
       </c>
@@ -6847,13 +6843,13 @@
         <v>353</v>
       </c>
       <c r="N119" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U119" s="2" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="120" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A120" s="2" t="s">
         <v>329</v>
       </c>
@@ -6870,7 +6866,7 @@
         <v>40</v>
       </c>
       <c r="G120" s="2" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="H120" s="2" t="s">
         <v>352</v>
@@ -6882,7 +6878,7 @@
         <v>3</v>
       </c>
       <c r="K120" s="3" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="L120" s="2" t="s">
         <v>352</v>
@@ -6891,10 +6887,10 @@
         <v>353</v>
       </c>
       <c r="N120" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="121" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="121" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A121" s="2" t="s">
         <v>330</v>
       </c>
@@ -6917,7 +6913,7 @@
         <v>4</v>
       </c>
       <c r="K121" s="2" t="s">
-        <v>604</v>
+        <v>596</v>
       </c>
       <c r="L121" s="2" t="s">
         <v>352</v>
@@ -6926,10 +6922,10 @@
         <v>353</v>
       </c>
       <c r="N121" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="122" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="122" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A122" s="2" t="s">
         <v>331</v>
       </c>
@@ -6952,7 +6948,7 @@
         <v>3</v>
       </c>
       <c r="K122" s="2" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="L122" s="2" t="s">
         <v>353</v>
@@ -6961,10 +6957,10 @@
         <v>352</v>
       </c>
       <c r="N122" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="123" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="123" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A123" s="2" t="s">
         <v>332</v>
       </c>
@@ -6996,10 +6992,10 @@
         <v>352</v>
       </c>
       <c r="N123" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="124" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="124" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A124" s="2" t="s">
         <v>333</v>
       </c>
@@ -7016,10 +7012,10 @@
         <v>71</v>
       </c>
       <c r="F124" s="2" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="G124" s="2" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="H124" s="2" t="s">
         <v>352</v>
@@ -7031,7 +7027,7 @@
         <v>4</v>
       </c>
       <c r="K124" s="3" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="L124" s="2" t="s">
         <v>352</v>
@@ -7040,10 +7036,10 @@
         <v>353</v>
       </c>
       <c r="N124" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="125" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="125" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A125" s="2" t="s">
         <v>334</v>
       </c>
@@ -7060,7 +7056,7 @@
         <v>73</v>
       </c>
       <c r="G125" s="2" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="H125" s="2" t="s">
         <v>352</v>
@@ -7072,7 +7068,7 @@
         <v>5</v>
       </c>
       <c r="K125" s="2" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="L125" s="2" t="s">
         <v>352</v>
@@ -7081,13 +7077,13 @@
         <v>353</v>
       </c>
       <c r="N125" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U125" s="2" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="126" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="126" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A126" s="2" t="s">
         <v>335</v>
       </c>
@@ -7104,7 +7100,7 @@
         <v>75</v>
       </c>
       <c r="G126" s="2" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="H126" s="2" t="s">
         <v>352</v>
@@ -7116,7 +7112,7 @@
         <v>6</v>
       </c>
       <c r="K126" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="L126" s="2" t="s">
         <v>352</v>
@@ -7125,10 +7121,10 @@
         <v>352</v>
       </c>
       <c r="N126" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="127" spans="1:21" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="127" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A127" s="2" t="s">
         <v>336</v>
       </c>
@@ -7157,13 +7153,13 @@
         <v>353</v>
       </c>
       <c r="N127" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U127" s="2" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="128" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A128" s="2" t="s">
         <v>337</v>
       </c>
@@ -7186,7 +7182,7 @@
         <v>6</v>
       </c>
       <c r="K128" s="2" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="L128" s="2" t="s">
         <v>352</v>
@@ -7195,10 +7191,10 @@
         <v>353</v>
       </c>
       <c r="N128" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="129" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="129" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A129" s="2" t="s">
         <v>338</v>
       </c>
@@ -7227,10 +7223,10 @@
         <v>353</v>
       </c>
       <c r="N129" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="130" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="130" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A130" s="2" t="s">
         <v>339</v>
       </c>
@@ -7247,7 +7243,7 @@
         <v>80</v>
       </c>
       <c r="G130" s="2" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="H130" s="2" t="s">
         <v>352</v>
@@ -7259,7 +7255,7 @@
         <v>4</v>
       </c>
       <c r="K130" s="2" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="L130" s="2" t="s">
         <v>352</v>
@@ -7268,10 +7264,10 @@
         <v>353</v>
       </c>
       <c r="N130" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="131" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="131" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A131" s="2" t="s">
         <v>340</v>
       </c>
@@ -7288,7 +7284,7 @@
         <v>81</v>
       </c>
       <c r="G131" s="2" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="H131" s="2" t="s">
         <v>352</v>
@@ -7300,7 +7296,7 @@
         <v>5</v>
       </c>
       <c r="K131" s="2" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="L131" s="2" t="s">
         <v>352</v>
@@ -7309,10 +7305,10 @@
         <v>353</v>
       </c>
       <c r="N131" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="132" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="132" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A132" s="2" t="s">
         <v>341</v>
       </c>
@@ -7329,10 +7325,10 @@
         <v>82</v>
       </c>
       <c r="F132" s="2" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="G132" s="2" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="H132" s="2" t="s">
         <v>352</v>
@@ -7344,7 +7340,7 @@
         <v>6</v>
       </c>
       <c r="K132" s="2" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="L132" s="2" t="s">
         <v>352</v>
@@ -7353,13 +7349,13 @@
         <v>353</v>
       </c>
       <c r="N132" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="P132" s="2" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="133" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="133" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A133" s="2" t="s">
         <v>342</v>
       </c>
@@ -7373,7 +7369,7 @@
         <v>105</v>
       </c>
       <c r="F133" s="10" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="G133" s="10"/>
       <c r="H133" s="2" t="s">
@@ -7386,7 +7382,7 @@
         <v>6</v>
       </c>
       <c r="K133" s="3" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="L133" s="2" t="s">
         <v>352</v>
@@ -7395,10 +7391,10 @@
         <v>353</v>
       </c>
       <c r="N133" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="134" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="134" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A134" s="2" t="s">
         <v>343</v>
       </c>
@@ -7416,7 +7412,7 @@
       </c>
       <c r="F134" s="10"/>
       <c r="G134" s="10" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="H134" s="2" t="s">
         <v>352</v>
@@ -7434,10 +7430,10 @@
         <v>353</v>
       </c>
       <c r="N134" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="135" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="135" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A135" s="2" t="s">
         <v>344</v>
       </c>
@@ -7457,7 +7453,7 @@
         <v>203</v>
       </c>
       <c r="G135" s="10" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="H135" s="2" t="s">
         <v>352</v>
@@ -7469,7 +7465,7 @@
         <v>3</v>
       </c>
       <c r="K135" s="3" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
       <c r="L135" s="2" t="s">
         <v>352</v>
@@ -7478,10 +7474,10 @@
         <v>353</v>
       </c>
       <c r="N135" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="136" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="136" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A136" s="2" t="s">
         <v>345</v>
       </c>
@@ -7498,7 +7494,7 @@
         <v>41</v>
       </c>
       <c r="G136" s="2" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="H136" s="2" t="s">
         <v>352</v>
@@ -7516,10 +7512,10 @@
         <v>353</v>
       </c>
       <c r="N136" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="137" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="137" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A137" s="2" t="s">
         <v>346</v>
       </c>
@@ -7542,7 +7538,7 @@
         <v>4</v>
       </c>
       <c r="K137" s="2" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="L137" s="2" t="s">
         <v>352</v>
@@ -7551,10 +7547,10 @@
         <v>353</v>
       </c>
       <c r="N137" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="138" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="138" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A138" s="2" t="s">
         <v>347</v>
       </c>
@@ -7580,13 +7576,13 @@
         <v>353</v>
       </c>
       <c r="N138" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U138" s="2" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="139" spans="1:21" ht="72" hidden="1" x14ac:dyDescent="0.3">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="139" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="A139" s="2" t="s">
         <v>348</v>
       </c>
@@ -7609,7 +7605,7 @@
         <v>7</v>
       </c>
       <c r="K139" s="3" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="L139" s="2" t="s">
         <v>352</v>
@@ -7618,13 +7614,13 @@
         <v>353</v>
       </c>
       <c r="N139" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="R139" s="2" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="140" spans="1:21" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="140" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A140" s="2" t="s">
         <v>349</v>
       </c>
@@ -7638,7 +7634,7 @@
         <v>6</v>
       </c>
       <c r="F140" s="2" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="H140" s="2" t="s">
         <v>352</v>
@@ -7650,7 +7646,7 @@
         <v>1</v>
       </c>
       <c r="K140" s="3" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="L140" s="2" t="s">
         <v>352</v>
@@ -7659,10 +7655,10 @@
         <v>352</v>
       </c>
       <c r="N140" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="141" spans="1:21" ht="72" hidden="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="141" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A141" s="2" t="s">
         <v>350</v>
       </c>
@@ -7685,7 +7681,7 @@
         <v>4</v>
       </c>
       <c r="K141" s="3" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="L141" s="3" t="s">
         <v>352</v>
@@ -7694,13 +7690,13 @@
         <v>353</v>
       </c>
       <c r="N141" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U141" s="2" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="142" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A142" s="2" t="s">
         <v>359</v>
       </c>
@@ -7711,7 +7707,7 @@
         <v>193</v>
       </c>
       <c r="E142" s="2" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="H142" s="2" t="s">
         <v>352</v>
@@ -7720,7 +7716,7 @@
         <v>360</v>
       </c>
       <c r="J142" s="2" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="L142" s="2" t="s">
         <v>353</v>
@@ -7729,167 +7725,167 @@
         <v>353</v>
       </c>
       <c r="N142" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="U142" s="12" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="143" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A143" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="B143" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="E143" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="H143" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="I143" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="J143" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="K143" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="L143" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="M143" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="N143" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="U143" s="2" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="144" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A144" s="2" t="s">
         <v>386</v>
       </c>
-      <c r="B143" s="2" t="s">
-        <v>392</v>
-      </c>
-      <c r="E143" s="2" t="s">
-        <v>393</v>
-      </c>
-      <c r="H143" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="I143" s="2" t="s">
+      <c r="B144" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="E144" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="H144" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="I144" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="K144" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="L144" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="M144" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="N144" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="U144" s="2" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="145" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A145" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="B145" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="E145" s="2" t="s">
         <v>394</v>
       </c>
-      <c r="J143" s="2" t="s">
-        <v>381</v>
-      </c>
-      <c r="K143" s="2" t="s">
+      <c r="H145" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="I145" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="K145" s="2" t="s">
         <v>442</v>
       </c>
-      <c r="L143" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="M143" s="2" t="s">
-        <v>353</v>
-      </c>
-      <c r="N143" s="2" t="s">
-        <v>438</v>
-      </c>
-      <c r="U143" s="2" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="144" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A144" s="2" t="s">
-        <v>387</v>
-      </c>
-      <c r="B144" s="2" t="s">
-        <v>392</v>
-      </c>
-      <c r="E144" s="2" t="s">
-        <v>389</v>
-      </c>
-      <c r="H144" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="I144" s="2" t="s">
+      <c r="L145" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="M145" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="N145" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="U145" s="2" t="s">
         <v>390</v>
-      </c>
-      <c r="K144" s="2" t="s">
-        <v>444</v>
-      </c>
-      <c r="L144" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="M144" s="2" t="s">
-        <v>353</v>
-      </c>
-      <c r="N144" s="2" t="s">
-        <v>438</v>
-      </c>
-      <c r="U144" s="2" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="145" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A145" s="2" t="s">
-        <v>388</v>
-      </c>
-      <c r="B145" s="2" t="s">
-        <v>392</v>
-      </c>
-      <c r="E145" s="2" t="s">
-        <v>395</v>
-      </c>
-      <c r="H145" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="I145" s="2" t="s">
-        <v>390</v>
-      </c>
-      <c r="K145" s="2" t="s">
-        <v>443</v>
-      </c>
-      <c r="L145" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="M145" s="2" t="s">
-        <v>353</v>
-      </c>
-      <c r="N145" s="2" t="s">
-        <v>438</v>
-      </c>
-      <c r="U145" s="2" t="s">
-        <v>391</v>
       </c>
     </row>
     <row r="146" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A146" s="2" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="E146" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="H146" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="I146" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="J146" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="K146" s="2" t="s">
+        <v>463</v>
+      </c>
+      <c r="L146" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="M146" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="N146" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="U146" s="2" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="147" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A147" s="2" t="s">
         <v>450</v>
       </c>
-      <c r="H146" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="I146" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="J146" s="2" t="s">
-        <v>445</v>
-      </c>
-      <c r="K146" s="2" t="s">
-        <v>464</v>
-      </c>
-      <c r="L146" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="M146" s="2" t="s">
-        <v>353</v>
-      </c>
-      <c r="N146" s="2" t="s">
-        <v>438</v>
-      </c>
-      <c r="U146" s="2" t="s">
+      <c r="B147" s="2" t="s">
         <v>391</v>
       </c>
-    </row>
-    <row r="147" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A147" s="2" t="s">
+      <c r="E147" s="2" t="s">
         <v>451</v>
       </c>
-      <c r="B147" s="2" t="s">
-        <v>392</v>
-      </c>
-      <c r="E147" s="2" t="s">
-        <v>452</v>
-      </c>
       <c r="H147" s="2" t="s">
         <v>352</v>
       </c>
       <c r="I147" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J147" s="2" t="s">
         <v>362</v>
       </c>
       <c r="K147" s="2" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="L147" s="2" t="s">
         <v>352</v>
@@ -7898,36 +7894,36 @@
         <v>353</v>
       </c>
       <c r="N147" s="2" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="148" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="148" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A148" s="2" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B148" s="2" t="s">
         <v>83</v>
       </c>
       <c r="D148" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="E148" s="2" t="s">
         <v>404</v>
       </c>
-      <c r="E148" s="2" t="s">
+      <c r="F148" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="H148" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="I148" s="2" t="s">
         <v>405</v>
       </c>
-      <c r="F148" s="2" t="s">
-        <v>533</v>
-      </c>
-      <c r="H148" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="I148" s="2" t="s">
+      <c r="J148" s="2" t="s">
         <v>406</v>
       </c>
-      <c r="J148" s="2" t="s">
-        <v>407</v>
-      </c>
       <c r="K148" s="2" t="s">
-        <v>592</v>
+        <v>588</v>
       </c>
       <c r="L148" s="2" t="s">
         <v>352</v>
@@ -7936,191 +7932,191 @@
         <v>353</v>
       </c>
       <c r="N148" s="2" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="149" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A149" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="B149" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="E149" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="H149" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="I149" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="K149" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="L149" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="M149" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="N149" s="2" t="s">
         <v>437</v>
       </c>
-    </row>
-    <row r="149" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A149" s="2" t="s">
-        <v>439</v>
-      </c>
-      <c r="B149" s="2" t="s">
-        <v>392</v>
-      </c>
-      <c r="E149" s="2" t="s">
-        <v>372</v>
-      </c>
-      <c r="H149" s="2" t="s">
-        <v>353</v>
-      </c>
-      <c r="I149" s="2" t="s">
-        <v>440</v>
-      </c>
-      <c r="K149" s="2" t="s">
-        <v>441</v>
-      </c>
-      <c r="L149" s="2" t="s">
-        <v>353</v>
-      </c>
-      <c r="M149" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="N149" s="2" t="s">
-        <v>438</v>
-      </c>
       <c r="U149" s="2" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="150" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A150" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="B150" s="2" t="s">
         <v>391</v>
       </c>
-    </row>
-    <row r="150" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A150" s="2" t="s">
+      <c r="E150" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="H150" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="I150" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="J150" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="K150" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="L150" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="M150" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="N150" s="2" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="151" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A151" s="2" t="s">
         <v>453</v>
       </c>
-      <c r="B150" s="2" t="s">
-        <v>392</v>
-      </c>
-      <c r="E150" s="2" t="s">
+      <c r="B151" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="E151" s="2" t="s">
         <v>457</v>
       </c>
-      <c r="H150" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="I150" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="J150" s="2" t="s">
-        <v>407</v>
-      </c>
-      <c r="K150" s="2" t="s">
+      <c r="H151" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="I151" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="J151" s="2" t="s">
+        <v>461</v>
+      </c>
+      <c r="K151" s="2" t="s">
         <v>466</v>
       </c>
-      <c r="L150" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="M150" s="2" t="s">
-        <v>353</v>
-      </c>
-      <c r="N150" s="2" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="151" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A151" s="2" t="s">
+      <c r="L151" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="M151" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="N151" s="2" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="152" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A152" s="2" t="s">
         <v>454</v>
       </c>
-      <c r="B151" s="2" t="s">
-        <v>392</v>
-      </c>
-      <c r="E151" s="2" t="s">
+      <c r="B152" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="E152" s="2" t="s">
         <v>458</v>
       </c>
-      <c r="H151" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="I151" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="J151" s="2" t="s">
+      <c r="H152" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="I152" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="J152" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="K152" s="2" t="s">
+        <v>467</v>
+      </c>
+      <c r="L152" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="M152" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="N152" s="2" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="153" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A153" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="B153" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="E153" s="2" t="s">
+        <v>459</v>
+      </c>
+      <c r="H153" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="I153" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="J153" s="2" t="s">
         <v>462</v>
       </c>
-      <c r="K151" s="2" t="s">
-        <v>467</v>
-      </c>
-      <c r="L151" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="M151" s="2" t="s">
-        <v>353</v>
-      </c>
-      <c r="N151" s="2" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="152" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A152" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="B152" s="2" t="s">
-        <v>392</v>
-      </c>
-      <c r="E152" s="2" t="s">
-        <v>459</v>
-      </c>
-      <c r="H152" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="I152" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="J152" s="2" t="s">
-        <v>446</v>
-      </c>
-      <c r="K152" s="2" t="s">
+      <c r="K153" s="2" t="s">
         <v>468</v>
       </c>
-      <c r="L152" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="M152" s="2" t="s">
-        <v>353</v>
-      </c>
-      <c r="N152" s="2" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="153" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A153" s="2" t="s">
-        <v>456</v>
-      </c>
-      <c r="B153" s="2" t="s">
-        <v>392</v>
-      </c>
-      <c r="E153" s="2" t="s">
+      <c r="L153" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="M153" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="N153" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="R153" s="2" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="154" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A154" s="2" t="s">
         <v>460</v>
       </c>
-      <c r="H153" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="I153" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="J153" s="2" t="s">
-        <v>463</v>
-      </c>
-      <c r="K153" s="2" t="s">
+      <c r="B154" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="E154" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="H154" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="I154" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="K154" s="2" t="s">
         <v>469</v>
       </c>
-      <c r="L153" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="M153" s="2" t="s">
-        <v>353</v>
-      </c>
-      <c r="N153" s="2" t="s">
-        <v>438</v>
-      </c>
-      <c r="R153" s="2" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="154" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A154" s="2" t="s">
-        <v>461</v>
-      </c>
-      <c r="B154" s="2" t="s">
-        <v>392</v>
-      </c>
-      <c r="E154" s="2" t="s">
-        <v>397</v>
-      </c>
-      <c r="H154" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="I154" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="K154" s="2" t="s">
-        <v>470</v>
-      </c>
       <c r="L154" s="2" t="s">
         <v>352</v>
       </c>
@@ -8128,24 +8124,24 @@
         <v>353</v>
       </c>
       <c r="N154" s="2" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="155" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="155" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A155" s="2" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="E155" s="2" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="H155" s="2" t="s">
         <v>352</v>
       </c>
       <c r="K155" s="2" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L155" s="2" t="s">
         <v>352</v>
@@ -8154,12 +8150,12 @@
         <v>353</v>
       </c>
       <c r="N155" s="2" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="156" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="156" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A156" s="2" t="s">
-        <v>584</v>
+        <v>580</v>
       </c>
       <c r="B156" s="2" t="s">
         <v>125</v>
@@ -8171,19 +8167,19 @@
         <v>139</v>
       </c>
       <c r="F156" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="H156" s="2" t="s">
         <v>352</v>
       </c>
       <c r="I156" s="2" t="s">
-        <v>585</v>
+        <v>581</v>
       </c>
       <c r="J156" s="2">
         <v>6</v>
       </c>
       <c r="K156" s="2" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="L156" s="2" t="s">
         <v>352</v>
@@ -8192,23 +8188,17 @@
         <v>353</v>
       </c>
       <c r="N156" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="R156" s="2" t="s">
-        <v>609</v>
+        <v>600</v>
       </c>
       <c r="U156" s="2" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V156" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <filterColumn colId="9">
-      <filters>
-        <filter val="2"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:V156" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N146">
     <sortCondition ref="E2:E146"/>
     <sortCondition ref="I2:I146"/>

</xml_diff>

<commit_message>
update of Tarsp Index
</commit_message>
<xml_diff>
--- a/src/sastadev/data/methods/TARSP_Index_Current.xlsx
+++ b/src/sastadev/data/methods/TARSP_Index_Current.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\jodijk\myprograms\python\sastacode\mysastadev\src\sastadev\data\methods\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{873004BA-7E8D-4739-91FC-DDCBED97027F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B81D29EC-E62B-41EF-A214-7A85DAC4B56C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -8262,7 +8262,7 @@
         <v>616</v>
       </c>
       <c r="L157" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="M157" s="2" t="s">
         <v>353</v>

</xml_diff>